<commit_message>
Updates to broken words not getting translated.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF33ADC-5EF9-492A-BA81-42F6272BB79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F293345-76D5-451A-8496-850233FEA76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14520" yWindow="4240" windowWidth="20960" windowHeight="13380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="506">
   <si>
     <t>interview</t>
   </si>
@@ -8458,20 +8458,63 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
-% if get_config("interview page pre"):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ get_config("interview page pre") }</t>
+      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list)) &gt; 0:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div style="float: right;"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action("interview_list_delete_all"), label=word("Eliminar todo"), size="md", color="danger", icon="trash-can", id_tag="al-delete-all-sessions") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
     </r>
     <r>
       <rPr>
@@ -8493,938 +8536,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
-Usa la acción de etiqueta </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:tag:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> para agregar o editar una descripción.
-**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">% endif
 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;nav aria-label="Page navigation"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if session_page &gt; 0:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Previo</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Next</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/ul&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/nav&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">You do not have any Easy Forms in progress.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list)) &gt; 0:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;div style="float: right;"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action("interview_list_delete_all"), label=word("Eliminar todo"), size="md", color="danger", icon="trash-can", id_tag="al-delete-all-sessions") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/div&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
-% if PAGE_SUBQUESTION:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ PAGE_SUBQUESTION }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Toque el título de un formulario para seguir trabajando en él o para descargar sus documentos completados.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if showifdef("limit_filename") or showifdef("search_keyword"):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ session_list_html(answers = find_matching_sessions(filenames={limit_filename} if limit_filename else None, keyword=search_keyword), filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;nav aria-label="Navegación de página"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if session_page &gt; 0:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Previous</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Próxima</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/ul&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/nav&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if showifdef("limit_filename") or showifdef("search_keyword"):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action("delete_results_action"), label=word("Borrar resultados de búsqueda"), size="md", color="secondary", icon="times-circle", id_tag="al-clear-search-results") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
     </r>
   </si>
   <si>
@@ -10258,296 +9371,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Sign in**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) or </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**create**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) an ILAO Easy Form account to **save your progress**.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Feedback, suggestions, or comments? </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**Let us know**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">){:target='_blank'}.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if nav.get_section() != None:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if current_context().question_id == None:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=word('^^edit^^ Edit answers'), color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif 'review screen' not in current_context().question_id:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=word('^^edit^^ Edit answers'), color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Iniciar sesión**]</t>
     </r>
     <r>
@@ -10730,6 +9553,1524 @@
       <t>% endif
 % endif
 % endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Sign in**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) or [**create**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) an ILAO Easy Form account to **save your progress**.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Feedback, suggestions, or comments? [**Let us know**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">){:target='_blank'}.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if nav.get_section() != None:
+% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
+% if current_context().question_id == None:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif 'review screen' not in current_context().question_id:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif
+% endif
+% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
+% if PAGE_SUBQUESTION:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ PAGE_SUBQUESTION }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Toque el título de un formulario para seguir trabajando en él o para descargar sus documentos completados.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if showifdef("limit_filename") or showifdef("search_keyword"):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ session_list_html(answers = find_matching_sessions(filenames={limit_filename} if limit_filename else None, keyword=search_keyword), filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;nav aria-label="Navegación de página"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if session_page &gt; 0:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Previo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Próximo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/ul&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/nav&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if showifdef("limit_filename") or showifdef("search_keyword"):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action("delete_results_action"), label=word("Borrar resultados de búsqueda"), size="md", color="secondary", icon="times-circle", id_tag="al-clear-search-results") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
+% if get_config("interview page pre"):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ get_config("interview page pre") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
+Usa la acción de etiqueta </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:tag:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para agregar o editar una descripción.
+**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;nav aria-label="Page navigation"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if session_page &gt; 0:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Previo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Próximo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/ul&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/nav&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">You do not have any Easy Forms in progress.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <t>4e55bf25f68974cec62059b2f730bfb9</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div id='nav-title-container' class='title-container'&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="al-logo"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;img src="/packagestatic/docassemble.ILAO/logo_white_30.svg" alt="Illinois Legal Aid Online"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="al-title"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="title-row-1"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ localized_metadata_text(all_variables(special='metadata'), 'title') }</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="title-row-2"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ "Home" }</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div id='nav-title-container' class='title-container'&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="al-logo"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;img src="/packagestatic/docassemble.ILAO/logo_white_30.svg" alt="Illinois Legal Aid Online"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="al-title"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="title-row-1"&gt;${ localized_metadata_text(all_variables(special='metadata'), 'title') }&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;div class="title-row-2"&gt;${ "Hogar" }&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/div&gt;</t>
     </r>
   </si>
 </sst>
@@ -11160,7 +11501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H158"/>
+  <dimension ref="A1:H159"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="57.453125" customWidth="1"/>
@@ -11311,19 +11652,19 @@
         <v>5</v>
       </c>
       <c r="D6" s="11" t="s">
+        <v>498</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>501</v>
-      </c>
       <c r="H6" s="4" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="225" customHeight="1" x14ac:dyDescent="0.35">
@@ -14521,7 +14862,7 @@
         <v>431</v>
       </c>
       <c r="H129" s="14" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
@@ -14547,7 +14888,7 @@
         <v>433</v>
       </c>
       <c r="H130" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
@@ -14573,7 +14914,7 @@
         <v>435</v>
       </c>
       <c r="H131" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="405" customHeight="1" x14ac:dyDescent="0.35">
@@ -14649,7 +14990,7 @@
         <v>441</v>
       </c>
       <c r="H134" s="4" t="s">
-        <v>491</v>
+        <v>501</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -14675,7 +15016,7 @@
         <v>443</v>
       </c>
       <c r="H135" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.35">
@@ -14725,7 +15066,7 @@
         <v>447</v>
       </c>
       <c r="H137" s="4" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -14853,7 +15194,7 @@
         <v>458</v>
       </c>
       <c r="H142" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
@@ -14879,7 +15220,7 @@
         <v>460</v>
       </c>
       <c r="H143" s="4" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -15165,7 +15506,7 @@
         <v>424</v>
       </c>
       <c r="H154" s="4" t="s">
-        <v>489</v>
+        <v>502</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
@@ -15188,10 +15529,10 @@
         <v>9</v>
       </c>
       <c r="G155" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="H155" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="156" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -15270,6 +15611,32 @@
       </c>
       <c r="H158" s="5" t="s">
         <v>373</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A159" s="11" t="s">
+        <v>407</v>
+      </c>
+      <c r="B159" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="C159" s="11">
+        <v>1</v>
+      </c>
+      <c r="D159" s="11" t="s">
+        <v>503</v>
+      </c>
+      <c r="E159" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F159" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G159" s="12" t="s">
+        <v>504</v>
+      </c>
+      <c r="H159" s="4" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Latest updates to ILAO framework basic questions, XLSX, and words.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE13B02-B1C4-490F-87B2-420D7CFA9D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314695A5-4BE1-444C-B9EF-E5C6D6FDFAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10820" yWindow="2590" windowWidth="25640" windowHeight="14670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2170,9 +2170,6 @@
     <t>Acepto los términos de uso y la política de privacidad.</t>
   </si>
   <si>
-    <t>No puedes continuar a menos que aceptes los términos de uso y la política de privacidad.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -11062,6 +11059,9 @@
 % endif
 % endif</t>
     </r>
+  </si>
+  <si>
+    <t>No puedes continuar a menos que aceptes los Términos de uso y la Política de privacidad.</t>
   </si>
 </sst>
 </file>
@@ -11512,16 +11512,16 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>8</v>
@@ -11530,24 +11530,24 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>8</v>
@@ -11556,119 +11556,119 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C4" s="5">
         <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C5" s="5">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="3" t="s">
         <v>302</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C6" s="5">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>479</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>480</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C7" s="5">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>382</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
@@ -11694,7 +11694,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
@@ -11712,15 +11712,15 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
@@ -11746,7 +11746,7 @@
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>14</v>
@@ -11767,12 +11767,12 @@
         <v>54</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>14</v>
@@ -11790,7 +11790,7 @@
         <v>9</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>224</v>
@@ -11798,7 +11798,7 @@
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>14</v>
@@ -11819,12 +11819,12 @@
         <v>58</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -11850,7 +11850,7 @@
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11868,15 +11868,15 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11902,7 +11902,7 @@
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11920,15 +11920,15 @@
         <v>9</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11954,7 +11954,7 @@
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -11972,15 +11972,15 @@
         <v>9</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -12006,7 +12006,7 @@
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -12024,15 +12024,15 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -12058,7 +12058,7 @@
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -12084,7 +12084,7 @@
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -12110,7 +12110,7 @@
     </row>
     <row r="25" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -12131,12 +12131,12 @@
         <v>42</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -12157,12 +12157,12 @@
         <v>44</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -12188,7 +12188,7 @@
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -12214,7 +12214,7 @@
     </row>
     <row r="29" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -12240,7 +12240,7 @@
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -12266,7 +12266,7 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -12287,12 +12287,12 @@
         <v>54</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -12318,7 +12318,7 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -12344,7 +12344,7 @@
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -12365,12 +12365,12 @@
         <v>60</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -12396,7 +12396,7 @@
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -12422,7 +12422,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12448,7 +12448,7 @@
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12474,7 +12474,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12500,7 +12500,7 @@
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12526,7 +12526,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12552,7 +12552,7 @@
     </row>
     <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12578,7 +12578,7 @@
     </row>
     <row r="43" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12604,7 +12604,7 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12630,7 +12630,7 @@
     </row>
     <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12651,12 +12651,12 @@
         <v>82</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12682,7 +12682,7 @@
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12708,7 +12708,7 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12734,7 +12734,7 @@
     </row>
     <row r="49" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12755,12 +12755,12 @@
         <v>90</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -12786,7 +12786,7 @@
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -12807,12 +12807,12 @@
         <v>94</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -12838,7 +12838,7 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -12864,7 +12864,7 @@
     </row>
     <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -12890,7 +12890,7 @@
     </row>
     <row r="55" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -12916,7 +12916,7 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -12942,7 +12942,7 @@
     </row>
     <row r="57" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -12968,7 +12968,7 @@
     </row>
     <row r="58" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>107</v>
@@ -12994,7 +12994,7 @@
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>110</v>
@@ -13020,7 +13020,7 @@
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>113</v>
@@ -13046,7 +13046,7 @@
     </row>
     <row r="61" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>113</v>
@@ -13072,7 +13072,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>113</v>
@@ -13098,7 +13098,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>113</v>
@@ -13124,7 +13124,7 @@
     </row>
     <row r="64" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>113</v>
@@ -13150,7 +13150,7 @@
     </row>
     <row r="65" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>113</v>
@@ -13176,7 +13176,7 @@
     </row>
     <row r="66" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>12</v>
@@ -13202,7 +13202,7 @@
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>12</v>
@@ -13228,7 +13228,7 @@
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>12</v>
@@ -13254,7 +13254,7 @@
     </row>
     <row r="69" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>12</v>
@@ -13280,7 +13280,7 @@
     </row>
     <row r="70" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>12</v>
@@ -13306,7 +13306,7 @@
     </row>
     <row r="71" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>12</v>
@@ -13332,7 +13332,7 @@
     </row>
     <row r="72" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>138</v>
@@ -13358,7 +13358,7 @@
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>138</v>
@@ -13384,7 +13384,7 @@
     </row>
     <row r="74" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>143</v>
@@ -13405,12 +13405,12 @@
         <v>145</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>143</v>
@@ -13434,9 +13434,9 @@
         <v>272</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>10</v>
@@ -13457,12 +13457,12 @@
         <v>149</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>150</v>
@@ -13488,7 +13488,7 @@
     </row>
     <row r="78" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>150</v>
@@ -13514,7 +13514,7 @@
     </row>
     <row r="79" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>155</v>
@@ -13540,7 +13540,7 @@
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>155</v>
@@ -13561,12 +13561,12 @@
         <v>159</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>160</v>
@@ -13592,7 +13592,7 @@
     </row>
     <row r="82" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>160</v>
@@ -13618,7 +13618,7 @@
     </row>
     <row r="83" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>160</v>
@@ -13644,7 +13644,7 @@
     </row>
     <row r="84" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>160</v>
@@ -13670,7 +13670,7 @@
     </row>
     <row r="85" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>160</v>
@@ -13691,12 +13691,12 @@
         <v>170</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>280</v>
+        <v>502</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>171</v>
@@ -13717,12 +13717,12 @@
         <v>173</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>171</v>
@@ -13743,12 +13743,12 @@
         <v>175</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>11</v>
@@ -13766,15 +13766,15 @@
         <v>9</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="H88" s="2" t="s">
         <v>387</v>
-      </c>
-      <c r="H88" s="2" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>11</v>
@@ -13795,12 +13795,12 @@
         <v>178</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>179</v>
@@ -13821,12 +13821,12 @@
         <v>181</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>179</v>
@@ -13847,12 +13847,12 @@
         <v>183</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>184</v>
@@ -13873,12 +13873,12 @@
         <v>186</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>184</v>
@@ -13899,12 +13899,12 @@
         <v>188</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>184</v>
@@ -13925,12 +13925,12 @@
         <v>190</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>184</v>
@@ -13951,12 +13951,12 @@
         <v>192</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>184</v>
@@ -13977,12 +13977,12 @@
         <v>194</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>184</v>
@@ -14003,12 +14003,12 @@
         <v>196</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>197</v>
@@ -14029,12 +14029,12 @@
         <v>199</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>197</v>
@@ -14055,12 +14055,12 @@
         <v>201</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>202</v>
@@ -14081,12 +14081,12 @@
         <v>204</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>202</v>
@@ -14104,15 +14104,15 @@
         <v>9</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H101" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>206</v>
@@ -14130,15 +14130,15 @@
         <v>9</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>208</v>
@@ -14164,7 +14164,7 @@
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>210</v>
@@ -14190,7 +14190,7 @@
     </row>
     <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>212</v>
@@ -14208,15 +14208,15 @@
         <v>9</v>
       </c>
       <c r="G105" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="H105" s="3" t="s">
         <v>378</v>
-      </c>
-      <c r="H105" s="3" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="106" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>212</v>
@@ -14237,12 +14237,12 @@
         <v>215</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>216</v>
@@ -14263,12 +14263,12 @@
         <v>218</v>
       </c>
       <c r="H107" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>219</v>
@@ -14289,12 +14289,12 @@
         <v>221</v>
       </c>
       <c r="H108" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="109" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>219</v>
@@ -14303,362 +14303,362 @@
         <v>1</v>
       </c>
       <c r="D109" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="E109" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F109" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G109" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="E109" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F109" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G109" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="H109" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C110" s="5">
         <v>0</v>
       </c>
       <c r="D110" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F110" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G110" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="E110" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F110" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G110" s="6" t="s">
-        <v>395</v>
-      </c>
       <c r="H110" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C111" s="5">
         <v>1</v>
       </c>
       <c r="D111" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="E111" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F111" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G111" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="E111" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F111" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G111" s="6" t="s">
-        <v>397</v>
-      </c>
       <c r="H111" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C112" s="5">
         <v>2</v>
       </c>
       <c r="D112" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="E112" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F112" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G112" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="E112" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F112" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G112" s="6" t="s">
-        <v>306</v>
-      </c>
       <c r="H112" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C113" s="5">
         <v>0</v>
       </c>
       <c r="D113" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="E113" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G113" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="E113" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F113" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G113" s="6" t="s">
+      <c r="H113" s="3" t="s">
         <v>309</v>
-      </c>
-      <c r="H113" s="3" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C114" s="5">
         <v>1</v>
       </c>
       <c r="D114" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G114" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="E114" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F114" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G114" s="6" t="s">
-        <v>312</v>
-      </c>
       <c r="H114" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C115" s="5">
         <v>2</v>
       </c>
       <c r="D115" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F115" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G115" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="E115" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F115" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G115" s="6" t="s">
-        <v>314</v>
-      </c>
       <c r="H115" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C116" s="5">
         <v>3</v>
       </c>
       <c r="D116" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="E116" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F116" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G116" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="E116" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F116" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G116" s="6" t="s">
-        <v>316</v>
-      </c>
       <c r="H116" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C117" s="5">
         <v>4</v>
       </c>
       <c r="D117" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="E117" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F117" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G117" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E117" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F117" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G117" s="6" t="s">
+      <c r="H117" s="3" t="s">
         <v>318</v>
-      </c>
-      <c r="H117" s="3" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C118" s="5">
         <v>5</v>
       </c>
       <c r="D118" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F118" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G118" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="E118" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G118" s="6" t="s">
+      <c r="H118" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="H118" s="3" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C119" s="5">
         <v>6</v>
       </c>
       <c r="D119" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="E119" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F119" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G119" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="E119" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F119" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G119" s="6" t="s">
+      <c r="H119" s="2" t="s">
         <v>324</v>
-      </c>
-      <c r="H119" s="2" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C120" s="5">
         <v>7</v>
       </c>
       <c r="D120" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G120" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="E120" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G120" s="6" t="s">
+      <c r="H120" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="H120" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C121" s="5">
         <v>0</v>
       </c>
       <c r="D121" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G121" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="E121" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F121" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G121" s="6" t="s">
-        <v>331</v>
-      </c>
       <c r="H121" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C122" s="5">
         <v>0</v>
       </c>
       <c r="D122" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G122" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="E122" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G122" s="6" t="s">
+      <c r="H122" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="H122" s="3" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>11</v>
@@ -14667,24 +14667,24 @@
         <v>0</v>
       </c>
       <c r="D123" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F123" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G123" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="E123" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G123" s="6" t="s">
+      <c r="H123" s="2" t="s">
         <v>337</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>11</v>
@@ -14693,24 +14693,24 @@
         <v>1</v>
       </c>
       <c r="D124" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="E124" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G124" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="E124" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F124" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G124" s="6" t="s">
-        <v>340</v>
-      </c>
       <c r="H124" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>11</v>
@@ -14719,24 +14719,24 @@
         <v>2</v>
       </c>
       <c r="D125" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G125" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="E125" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F125" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G125" s="6" t="s">
+      <c r="H125" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>11</v>
@@ -14757,192 +14757,192 @@
         <v>178</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="B127" s="5" t="s">
         <v>410</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>411</v>
       </c>
       <c r="C127" s="5">
         <v>0</v>
       </c>
       <c r="D127" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F127" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G127" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="E127" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G127" s="6" t="s">
-        <v>413</v>
-      </c>
       <c r="H127" s="8" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="B128" s="5" t="s">
         <v>410</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>411</v>
       </c>
       <c r="C128" s="5">
         <v>1</v>
       </c>
       <c r="D128" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G128" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="E128" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G128" s="6" t="s">
-        <v>415</v>
-      </c>
       <c r="H128" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="B129" s="5" t="s">
         <v>410</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>411</v>
       </c>
       <c r="C129" s="5">
         <v>2</v>
       </c>
       <c r="D129" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G129" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="E129" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G129" s="6" t="s">
-        <v>417</v>
-      </c>
       <c r="H129" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C130" s="5">
         <v>0</v>
       </c>
       <c r="D130" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G130" s="6" t="s">
         <v>418</v>
-      </c>
-      <c r="E130" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G130" s="6" t="s">
-        <v>419</v>
       </c>
       <c r="H130" s="7"/>
     </row>
     <row r="131" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C131" s="5">
         <v>1</v>
       </c>
       <c r="D131" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G131" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="E131" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G131" s="6" t="s">
-        <v>421</v>
-      </c>
       <c r="H131" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C132" s="5">
         <v>2</v>
       </c>
       <c r="D132" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G132" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="E132" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G132" s="6" t="s">
-        <v>423</v>
-      </c>
       <c r="H132" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="133" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C133" s="5">
         <v>3</v>
       </c>
       <c r="D133" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="E133" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F133" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G133" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="E133" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F133" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G133" s="6" t="s">
-        <v>425</v>
-      </c>
       <c r="H133" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>171</v>
@@ -14951,22 +14951,22 @@
         <v>0</v>
       </c>
       <c r="D134" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G134" s="6" t="s">
         <v>426</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F134" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G134" s="6" t="s">
-        <v>427</v>
       </c>
       <c r="H134" s="7"/>
     </row>
     <row r="135" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>171</v>
@@ -14975,24 +14975,24 @@
         <v>1</v>
       </c>
       <c r="D135" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="E135" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F135" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G135" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="E135" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F135" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G135" s="6" t="s">
-        <v>429</v>
-      </c>
       <c r="H135" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>171</v>
@@ -15001,24 +15001,24 @@
         <v>2</v>
       </c>
       <c r="D136" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F136" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G136" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="E136" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F136" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G136" s="6" t="s">
-        <v>431</v>
-      </c>
       <c r="H136" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>171</v>
@@ -15027,24 +15027,24 @@
         <v>3</v>
       </c>
       <c r="D137" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F137" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G137" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="E137" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F137" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G137" s="6" t="s">
-        <v>433</v>
-      </c>
       <c r="H137" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>171</v>
@@ -15053,369 +15053,369 @@
         <v>4</v>
       </c>
       <c r="D138" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="E138" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F138" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G138" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="E138" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F138" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G138" s="6" t="s">
-        <v>435</v>
-      </c>
       <c r="H138" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C139" s="5">
         <v>0</v>
       </c>
       <c r="D139" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G139" s="6" t="s">
         <v>437</v>
-      </c>
-      <c r="E139" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G139" s="6" t="s">
-        <v>438</v>
       </c>
       <c r="H139" s="7"/>
     </row>
     <row r="140" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C140" s="5">
         <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F140" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G140" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="E140" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G140" s="6" t="s">
-        <v>440</v>
-      </c>
       <c r="H140" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C141" s="5">
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G141" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="E141" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G141" s="6" t="s">
-        <v>442</v>
-      </c>
       <c r="H141" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C142" s="5">
         <v>0</v>
       </c>
       <c r="D142" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G142" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="E142" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G142" s="6" t="s">
-        <v>445</v>
-      </c>
       <c r="H142" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C143" s="5">
         <v>1</v>
       </c>
       <c r="D143" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="E143" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F143" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G143" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="E143" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G143" s="6" t="s">
-        <v>447</v>
-      </c>
       <c r="H143" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C144" s="5">
         <v>2</v>
       </c>
       <c r="D144" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="E144" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G144" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="E144" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F144" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G144" s="6" t="s">
-        <v>449</v>
-      </c>
       <c r="H144" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C145" s="5">
         <v>0</v>
       </c>
       <c r="D145" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E145" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F145" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G145" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="E145" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G145" s="6" t="s">
-        <v>451</v>
-      </c>
       <c r="H145" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A146" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C146" s="5">
         <v>1</v>
       </c>
       <c r="D146" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="E146" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F146" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G146" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="E146" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G146" s="6" t="s">
-        <v>453</v>
-      </c>
       <c r="H146" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C147" s="5">
         <v>2</v>
       </c>
       <c r="D147" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="E147" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F147" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G147" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="E147" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G147" s="6" t="s">
-        <v>455</v>
-      </c>
       <c r="H147" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C148" s="5">
         <v>0</v>
       </c>
       <c r="D148" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="E148" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F148" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G148" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="E148" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F148" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G148" s="6" t="s">
-        <v>458</v>
-      </c>
       <c r="H148" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C149" s="5">
         <v>0</v>
       </c>
       <c r="D149" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="E149" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F149" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G149" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="E149" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F149" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G149" s="6" t="s">
-        <v>409</v>
-      </c>
       <c r="H149" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A150" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C150" s="5">
         <v>1</v>
       </c>
       <c r="D150" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="E150" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F150" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G150" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="E150" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F150" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G150" s="6" t="s">
-        <v>348</v>
-      </c>
       <c r="H150" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A151" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C151" s="5">
         <v>0</v>
       </c>
       <c r="D151" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="E151" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F151" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G151" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="E151" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G151" s="6" t="s">
-        <v>351</v>
-      </c>
       <c r="H151" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A152" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C152" s="5">
         <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>8</v>
@@ -15424,24 +15424,24 @@
         <v>9</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A153" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C153" s="5">
         <v>2</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E153" s="5" t="s">
         <v>8</v>
@@ -15450,93 +15450,93 @@
         <v>9</v>
       </c>
       <c r="G153" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="H153" s="2" t="s">
         <v>477</v>
-      </c>
-      <c r="H153" s="2" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C154" s="5">
         <v>0</v>
       </c>
       <c r="D154" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="E154" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G154" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="E154" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F154" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G154" s="6" t="s">
+      <c r="H154" s="2" t="s">
         <v>356</v>
-      </c>
-      <c r="H154" s="2" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C155" s="5">
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G155" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="E155" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F155" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G155" s="6" t="s">
+      <c r="H155" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="H155" s="3" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C156" s="5">
         <v>2</v>
       </c>
       <c r="D156" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="E156" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G156" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="E156" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F156" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G156" s="6" t="s">
+      <c r="H156" s="3" t="s">
         <v>362</v>
-      </c>
-      <c r="H156" s="3" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A157" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B157" s="5" t="s">
         <v>216</v>
@@ -15545,19 +15545,19 @@
         <v>1</v>
       </c>
       <c r="D157" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="E157" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G157" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="E157" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G157" s="6" t="s">
+      <c r="H157" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="H157" s="2" t="s">
-        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates for handling translations for send_button_html
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314695A5-4BE1-444C-B9EF-E5C6D6FDFAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6CFD3BD-182A-436B-8833-0F8E9E13D8F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10820" yWindow="2590" windowWidth="25640" windowHeight="14670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4550" yWindow="6420" windowWidth="31530" windowHeight="13220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="505">
   <si>
     <t>interview</t>
   </si>
@@ -1592,10 +1592,6 @@
   </si>
   <si>
     <t>d484d53c764a714afd0df2fc5b87e81e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Almost done
-</t>
   </si>
   <si>
     <t>ab4c437676f0fc391a48e8c120360d63</t>
@@ -2164,64 +2160,7 @@
     </r>
   </si>
   <si>
-    <t>Para continuar, debes aceptar los términos de uso y la política de privacidad.</t>
-  </si>
-  <si>
     <t>Acepto los términos de uso y la política de privacidad.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Si tiene preguntas o inquietudes sobre su problema legal y desea asesoría legal, debe hablar con un abogado.
-Utilice </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**Obtenga ayuda legal**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://www.illinoislegalaid.org/get-legal-help</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) para encontrar servicios legales gratuitos o de bajo costo en su área.</t>
-    </r>
   </si>
   <si>
     <t>Reiniciar</t>
@@ -2585,9 +2524,6 @@
     <t>**PLACEHOLDER - ¿Qué significa firmar los formularios?**</t>
   </si>
   <si>
-    <t>Casi listo</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -2613,9 +2549,6 @@
     </r>
   </si>
   <si>
-    <t>Envía una copia de tus formularios a tu correo electrónico.</t>
-  </si>
-  <si>
     <t>Block_3</t>
   </si>
   <si>
@@ -3246,88 +3179,6 @@
   <si>
     <t xml:space="preserve">Hubo un error
 </t>
-  </si>
-  <si>
-    <t>0eee3878fde923571843f5b8b058d205</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">We ran into an error when we tried to load this screen.
-You can try one of these steps to recover your work:
-* Click **Back** and try again,
-* Visit the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**ILAO Form Library**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://www.illinoislegalaid.org/form-library</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) and try another Easy Form.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ collapse_template(al_formatted_error_message) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
   </si>
   <si>
     <t>fef46e5063ce3dc78b8ae64fa474241d</t>
@@ -3870,9 +3721,6 @@
   </si>
   <si>
     <t>palabras verdes</t>
-  </si>
-  <si>
-    <t>Send a copy of your forms to your email</t>
   </si>
   <si>
     <t>easy forms</t>
@@ -5213,54 +5061,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Se produjo un error al intentar cargar esta pantalla.
-Puedes intentar uno de estos pasos para recuperar tu trabajo:
-* Haz clic en **Atrás** y vuelve a intentarlo,
-* Visita la [**Biblioteca de formularios de ILAO**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://www.illinoislegalaid.org/form-library</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) y prueba otro Formulario Fácile.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ collapse_template(al_formatted_error_message) }</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <b/>
         <sz val="11"/>
         <color rgb="FF0000FF"/>
@@ -11062,6 +10862,211 @@
   </si>
   <si>
     <t>No puedes continuar a menos que aceptes los Términos de uso y la Política de privacidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send a copy of your forms to your email
+</t>
+  </si>
+  <si>
+    <t>casi listo</t>
+  </si>
+  <si>
+    <t>almost done</t>
+  </si>
+  <si>
+    <t>0c92f52412da85628dc1abd321df08f0</t>
+  </si>
+  <si>
+    <r>
+      <t>We ran into an error when we tried to load this screen.
+You can try one of these steps to recover your work:
+* Click **Back** and try again,
+* [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:comment-dots:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> **Tell us what happened**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url , easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>){target="_blank"}, or
+* Visit the [**ILAO Form Library**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.illinoislegalaid.org/form-library</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) and try another Easy Form.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ collapse_template(al_formatted_error_message) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Se produjo un error al intentar cargar esta pantalla.
+Puedes intentar uno de estos pasos para recuperar tu trabajo:
+* Haz clic en **Atrás** y vuelve a intentarlo,
+* [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url , easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
+* Visita la [**Biblioteca de formularios de ILAO**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.illinoislegalaid.org/form-library</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) y prueba otro Formulario Fácile.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ collapse_template(al_formatted_error_message) }</t>
+    </r>
+  </si>
+  <si>
+    <t>Para continuar, debes aceptar los [**términos de uso**](https://es.illinoislegalaid.org/about/terms-of-use) y la [**política de privacidad**](https://www.illinoislegalaid.org/about/privacy-policy).</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Si tiene preguntas o inquietudes sobre su problema legal y desea asesoría legal, debe hablar con un abogado.
+Utilice [**Obtenga ayuda legal**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/get-legal-help</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) para encontrar servicios legales gratuitos o de bajo costo en su área.</t>
+    </r>
+  </si>
+  <si>
+    <t>Envía una copia de tus formularios a tu correo electrónico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address line 2
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZIP code
+</t>
   </si>
 </sst>
 </file>
@@ -11512,16 +11517,16 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>8</v>
@@ -11530,24 +11535,24 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>8</v>
@@ -11556,24 +11561,24 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C4" s="5">
         <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11582,24 +11587,24 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C5" s="5">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>8</v>
@@ -11608,24 +11613,24 @@
         <v>9</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C6" s="5">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>8</v>
@@ -11634,24 +11639,24 @@
         <v>9</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>479</v>
+        <v>470</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C7" s="5">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11660,15 +11665,15 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
@@ -11689,12 +11694,12 @@
         <v>16</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
@@ -11712,15 +11717,15 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
@@ -11741,12 +11746,12 @@
         <v>19</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>14</v>
@@ -11767,12 +11772,12 @@
         <v>54</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>14</v>
@@ -11790,15 +11795,15 @@
         <v>9</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>14</v>
@@ -11819,12 +11824,12 @@
         <v>58</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -11845,12 +11850,12 @@
         <v>24</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11868,15 +11873,15 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11897,12 +11902,12 @@
         <v>27</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11920,15 +11925,15 @@
         <v>9</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11949,12 +11954,12 @@
         <v>30</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -11972,15 +11977,15 @@
         <v>9</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -12001,12 +12006,12 @@
         <v>33</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -12024,15 +12029,15 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -12053,12 +12058,12 @@
         <v>36</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -12079,12 +12084,12 @@
         <v>38</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -12105,12 +12110,12 @@
         <v>40</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -12131,12 +12136,12 @@
         <v>42</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -12157,12 +12162,12 @@
         <v>44</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -12183,12 +12188,12 @@
         <v>46</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -12209,12 +12214,12 @@
         <v>48</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -12235,12 +12240,12 @@
         <v>50</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -12261,12 +12266,12 @@
         <v>52</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -12287,12 +12292,12 @@
         <v>54</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -12313,12 +12318,12 @@
         <v>56</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -12339,12 +12344,12 @@
         <v>58</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -12365,12 +12370,12 @@
         <v>60</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -12391,12 +12396,12 @@
         <v>62</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -12417,12 +12422,12 @@
         <v>64</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12443,12 +12448,12 @@
         <v>66</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12469,12 +12474,12 @@
         <v>68</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12495,12 +12500,12 @@
         <v>70</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12521,12 +12526,12 @@
         <v>72</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12547,12 +12552,12 @@
         <v>74</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12573,12 +12578,12 @@
         <v>76</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12599,12 +12604,12 @@
         <v>78</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12625,12 +12630,12 @@
         <v>80</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12651,12 +12656,12 @@
         <v>82</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12677,12 +12682,12 @@
         <v>84</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12703,12 +12708,12 @@
         <v>86</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12729,12 +12734,12 @@
         <v>88</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12755,12 +12760,12 @@
         <v>90</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -12781,12 +12786,12 @@
         <v>92</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -12807,12 +12812,12 @@
         <v>94</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -12833,12 +12838,12 @@
         <v>96</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -12859,12 +12864,12 @@
         <v>98</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -12885,12 +12890,12 @@
         <v>100</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -12911,12 +12916,12 @@
         <v>102</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -12937,12 +12942,12 @@
         <v>104</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -12963,12 +12968,12 @@
         <v>106</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>107</v>
@@ -12989,12 +12994,12 @@
         <v>109</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>110</v>
@@ -13015,12 +13020,12 @@
         <v>112</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>113</v>
@@ -13041,12 +13046,12 @@
         <v>115</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>113</v>
@@ -13072,7 +13077,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>113</v>
@@ -13093,12 +13098,12 @@
         <v>119</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>113</v>
@@ -13124,7 +13129,7 @@
     </row>
     <row r="64" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>113</v>
@@ -13145,12 +13150,12 @@
         <v>123</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>113</v>
@@ -13171,12 +13176,12 @@
         <v>125</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>12</v>
@@ -13197,12 +13202,12 @@
         <v>127</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>12</v>
@@ -13223,12 +13228,12 @@
         <v>129</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>12</v>
@@ -13249,12 +13254,12 @@
         <v>131</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>12</v>
@@ -13275,12 +13280,12 @@
         <v>133</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>12</v>
@@ -13301,12 +13306,12 @@
         <v>135</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>12</v>
@@ -13327,12 +13332,12 @@
         <v>137</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>138</v>
@@ -13353,12 +13358,12 @@
         <v>140</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>138</v>
@@ -13379,12 +13384,12 @@
         <v>142</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>143</v>
@@ -13405,12 +13410,12 @@
         <v>145</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>462</v>
+        <v>453</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>143</v>
@@ -13431,12 +13436,12 @@
         <v>147</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>10</v>
@@ -13457,12 +13462,12 @@
         <v>149</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>461</v>
+        <v>452</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>150</v>
@@ -13483,12 +13488,12 @@
         <v>152</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>150</v>
@@ -13509,12 +13514,12 @@
         <v>154</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>155</v>
@@ -13535,12 +13540,12 @@
         <v>157</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>155</v>
@@ -13561,12 +13566,12 @@
         <v>159</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>160</v>
@@ -13587,12 +13592,12 @@
         <v>162</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>160</v>
@@ -13613,12 +13618,12 @@
         <v>164</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>160</v>
@@ -13638,13 +13643,13 @@
       <c r="G83" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="H83" s="3" t="s">
-        <v>278</v>
+      <c r="H83" s="2" t="s">
+        <v>500</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>160</v>
@@ -13665,12 +13670,12 @@
         <v>168</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>160</v>
@@ -13691,12 +13696,12 @@
         <v>170</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>171</v>
@@ -13717,12 +13722,12 @@
         <v>173</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>280</v>
+        <v>501</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>171</v>
@@ -13743,12 +13748,12 @@
         <v>175</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>11</v>
@@ -13766,15 +13771,15 @@
         <v>9</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>11</v>
@@ -13795,12 +13800,12 @@
         <v>178</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>179</v>
@@ -13821,12 +13826,12 @@
         <v>181</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>179</v>
@@ -13847,12 +13852,12 @@
         <v>183</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>184</v>
@@ -13873,12 +13878,12 @@
         <v>186</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>184</v>
@@ -13899,12 +13904,12 @@
         <v>188</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>184</v>
@@ -13925,12 +13930,12 @@
         <v>190</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>184</v>
@@ -13951,12 +13956,12 @@
         <v>192</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>184</v>
@@ -13977,12 +13982,12 @@
         <v>194</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>184</v>
@@ -14003,12 +14008,12 @@
         <v>196</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>197</v>
@@ -14029,12 +14034,12 @@
         <v>199</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>197</v>
@@ -14055,12 +14060,12 @@
         <v>201</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>202</v>
@@ -14078,15 +14083,15 @@
         <v>9</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>204</v>
+        <v>496</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>202</v>
@@ -14095,85 +14100,85 @@
         <v>1</v>
       </c>
       <c r="D101" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A102" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="B102" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F101" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G101" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
       </c>
       <c r="D102" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G102" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A103" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="B103" s="5" t="s">
         <v>207</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F102" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G102" s="6" t="s">
-        <v>376</v>
-      </c>
-      <c r="H102" s="3" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A103" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>208</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
       </c>
       <c r="D103" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F103" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G103" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A104" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="B104" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F103" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G103" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="H103" s="3" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A104" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>210</v>
       </c>
       <c r="C104" s="5">
         <v>0</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>8</v>
@@ -14182,24 +14187,24 @@
         <v>9</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>123</v>
+        <v>504</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C105" s="5">
         <v>0</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>8</v>
@@ -14208,102 +14213,102 @@
         <v>9</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
     </row>
     <row r="106" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C106" s="5">
         <v>1</v>
       </c>
       <c r="D106" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="E106" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G106" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="E106" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F106" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G106" s="6" t="s">
-        <v>215</v>
-      </c>
       <c r="H106" s="3" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C107" s="5">
         <v>2</v>
       </c>
       <c r="D107" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E107" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F107" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G107" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="E107" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F107" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G107" s="6" t="s">
-        <v>218</v>
-      </c>
       <c r="H107" s="2" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C108" s="5">
         <v>0</v>
       </c>
       <c r="D108" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E108" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F108" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G108" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="E108" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F108" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G108" s="6" t="s">
-        <v>221</v>
-      </c>
       <c r="H108" s="3" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="109" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C109" s="5">
         <v>1</v>
       </c>
       <c r="D109" s="5" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>8</v>
@@ -14312,24 +14317,24 @@
         <v>9</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C110" s="5">
         <v>0</v>
       </c>
       <c r="D110" s="5" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>8</v>
@@ -14338,24 +14343,24 @@
         <v>9</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C111" s="5">
         <v>1</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>8</v>
@@ -14364,24 +14369,24 @@
         <v>9</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>398</v>
+        <v>390</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C112" s="5">
         <v>2</v>
       </c>
       <c r="D112" s="5" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E112" s="5" t="s">
         <v>8</v>
@@ -14390,24 +14395,24 @@
         <v>9</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="H112" s="2" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C113" s="5">
         <v>0</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>8</v>
@@ -14416,24 +14421,24 @@
         <v>9</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C114" s="5">
         <v>1</v>
       </c>
       <c r="D114" s="5" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E114" s="5" t="s">
         <v>8</v>
@@ -14442,24 +14447,24 @@
         <v>9</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C115" s="5">
         <v>2</v>
       </c>
       <c r="D115" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="E115" s="5" t="s">
         <v>8</v>
@@ -14468,24 +14473,24 @@
         <v>9</v>
       </c>
       <c r="G115" s="6" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="H115" s="2" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C116" s="5">
         <v>3</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="E116" s="5" t="s">
         <v>8</v>
@@ -14494,24 +14499,24 @@
         <v>9</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C117" s="5">
         <v>4</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="E117" s="5" t="s">
         <v>8</v>
@@ -14520,24 +14525,24 @@
         <v>9</v>
       </c>
       <c r="G117" s="6" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C118" s="5">
         <v>5</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>8</v>
@@ -14546,24 +14551,24 @@
         <v>9</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C119" s="5">
         <v>6</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>8</v>
@@ -14572,24 +14577,24 @@
         <v>9</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="H119" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C120" s="5">
         <v>7</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>8</v>
@@ -14598,24 +14603,24 @@
         <v>9</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="H120" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C121" s="5">
         <v>0</v>
       </c>
       <c r="D121" s="5" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="E121" s="5" t="s">
         <v>8</v>
@@ -14624,24 +14629,24 @@
         <v>9</v>
       </c>
       <c r="G121" s="6" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="C122" s="5">
         <v>0</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>8</v>
@@ -14650,15 +14655,15 @@
         <v>9</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>11</v>
@@ -14667,7 +14672,7 @@
         <v>0</v>
       </c>
       <c r="D123" s="5" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>8</v>
@@ -14676,15 +14681,15 @@
         <v>9</v>
       </c>
       <c r="G123" s="6" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="H123" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="124" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.35">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>11</v>
@@ -14693,7 +14698,7 @@
         <v>1</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>338</v>
+        <v>497</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>8</v>
@@ -14702,15 +14707,15 @@
         <v>9</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>339</v>
+        <v>498</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>403</v>
+        <v>499</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>11</v>
@@ -14719,7 +14724,7 @@
         <v>2</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="E125" s="5" t="s">
         <v>8</v>
@@ -14728,15 +14733,15 @@
         <v>9</v>
       </c>
       <c r="G125" s="6" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="H125" s="2" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>11</v>
@@ -14757,21 +14762,21 @@
         <v>178</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="C127" s="5">
         <v>0</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="E127" s="5" t="s">
         <v>8</v>
@@ -14780,24 +14785,24 @@
         <v>9</v>
       </c>
       <c r="G127" s="6" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="C128" s="5">
         <v>1</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="E128" s="5" t="s">
         <v>8</v>
@@ -14806,24 +14811,24 @@
         <v>9</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
       <c r="H128" s="2" t="s">
-        <v>471</v>
+        <v>462</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="C129" s="5">
         <v>2</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="E129" s="5" t="s">
         <v>8</v>
@@ -14832,24 +14837,24 @@
         <v>9</v>
       </c>
       <c r="G129" s="6" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>473</v>
+        <v>464</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C130" s="5">
         <v>0</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="E130" s="5" t="s">
         <v>8</v>
@@ -14858,22 +14863,22 @@
         <v>9</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="H130" s="7"/>
     </row>
     <row r="131" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C131" s="5">
         <v>1</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>8</v>
@@ -14882,24 +14887,24 @@
         <v>9</v>
       </c>
       <c r="G131" s="6" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="H131" s="2" t="s">
-        <v>469</v>
+        <v>460</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C132" s="5">
         <v>2</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="E132" s="5" t="s">
         <v>8</v>
@@ -14908,24 +14913,24 @@
         <v>9</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="133" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C133" s="5">
         <v>3</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>8</v>
@@ -14934,15 +14939,15 @@
         <v>9</v>
       </c>
       <c r="G133" s="6" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>171</v>
@@ -14951,7 +14956,7 @@
         <v>0</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="E134" s="5" t="s">
         <v>8</v>
@@ -14960,13 +14965,13 @@
         <v>9</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="H134" s="7"/>
     </row>
     <row r="135" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>171</v>
@@ -14975,7 +14980,7 @@
         <v>1</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>8</v>
@@ -14984,15 +14989,15 @@
         <v>9</v>
       </c>
       <c r="G135" s="6" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="H135" s="2" t="s">
-        <v>470</v>
+        <v>461</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>171</v>
@@ -15001,7 +15006,7 @@
         <v>2</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>8</v>
@@ -15010,15 +15015,15 @@
         <v>9</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>460</v>
+        <v>451</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>171</v>
@@ -15027,7 +15032,7 @@
         <v>3</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>8</v>
@@ -15036,15 +15041,15 @@
         <v>9</v>
       </c>
       <c r="G137" s="6" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>458</v>
+        <v>449</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>171</v>
@@ -15053,7 +15058,7 @@
         <v>4</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>8</v>
@@ -15062,24 +15067,24 @@
         <v>9</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>459</v>
+        <v>450</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="C139" s="5">
         <v>0</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>8</v>
@@ -15088,22 +15093,22 @@
         <v>9</v>
       </c>
       <c r="G139" s="6" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="H139" s="7"/>
     </row>
     <row r="140" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="C140" s="5">
         <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>438</v>
+        <v>429</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>8</v>
@@ -15112,24 +15117,24 @@
         <v>9</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>439</v>
+        <v>430</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="C141" s="5">
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>8</v>
@@ -15138,24 +15143,24 @@
         <v>9</v>
       </c>
       <c r="G141" s="6" t="s">
-        <v>441</v>
+        <v>432</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>475</v>
+        <v>466</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="C142" s="5">
         <v>0</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>443</v>
+        <v>434</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>8</v>
@@ -15164,24 +15169,24 @@
         <v>9</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>444</v>
+        <v>435</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>468</v>
+        <v>459</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="C143" s="5">
         <v>1</v>
       </c>
       <c r="D143" s="5" t="s">
-        <v>445</v>
+        <v>436</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>8</v>
@@ -15190,24 +15195,24 @@
         <v>9</v>
       </c>
       <c r="G143" s="6" t="s">
-        <v>446</v>
+        <v>437</v>
       </c>
       <c r="H143" s="2" t="s">
-        <v>467</v>
+        <v>458</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="C144" s="5">
         <v>2</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>447</v>
+        <v>438</v>
       </c>
       <c r="E144" s="5" t="s">
         <v>8</v>
@@ -15216,24 +15221,24 @@
         <v>9</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>448</v>
+        <v>439</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>466</v>
+        <v>457</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C145" s="5">
         <v>0</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>449</v>
+        <v>440</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>8</v>
@@ -15242,24 +15247,24 @@
         <v>9</v>
       </c>
       <c r="G145" s="6" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
       <c r="H145" s="2" t="s">
-        <v>465</v>
+        <v>456</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A146" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C146" s="5">
         <v>1</v>
       </c>
       <c r="D146" s="5" t="s">
-        <v>451</v>
+        <v>442</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>8</v>
@@ -15268,24 +15273,24 @@
         <v>9</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>452</v>
+        <v>443</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>464</v>
+        <v>455</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="5" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C147" s="5">
         <v>2</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>8</v>
@@ -15294,24 +15299,24 @@
         <v>9</v>
       </c>
       <c r="G147" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="H147" s="2" t="s">
         <v>454</v>
-      </c>
-      <c r="H147" s="2" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>455</v>
+        <v>446</v>
       </c>
       <c r="C148" s="5">
         <v>0</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>456</v>
+        <v>447</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>8</v>
@@ -15320,24 +15325,24 @@
         <v>9</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>457</v>
+        <v>448</v>
       </c>
       <c r="H148" s="2" t="s">
-        <v>457</v>
+        <v>448</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C149" s="5">
         <v>0</v>
       </c>
       <c r="D149" s="5" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>8</v>
@@ -15346,24 +15351,24 @@
         <v>9</v>
       </c>
       <c r="G149" s="6" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A150" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="C150" s="5">
         <v>1</v>
       </c>
       <c r="D150" s="5" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>8</v>
@@ -15372,24 +15377,24 @@
         <v>9</v>
       </c>
       <c r="G150" s="6" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A151" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C151" s="5">
         <v>0</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="E151" s="5" t="s">
         <v>8</v>
@@ -15398,24 +15403,24 @@
         <v>9</v>
       </c>
       <c r="G151" s="6" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A152" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C152" s="5">
         <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>8</v>
@@ -15424,24 +15429,24 @@
         <v>9</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A153" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="C153" s="5">
         <v>2</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="E153" s="5" t="s">
         <v>8</v>
@@ -15450,24 +15455,24 @@
         <v>9</v>
       </c>
       <c r="G153" s="6" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C154" s="5">
         <v>0</v>
       </c>
       <c r="D154" s="5" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="E154" s="5" t="s">
         <v>8</v>
@@ -15476,24 +15481,24 @@
         <v>9</v>
       </c>
       <c r="G154" s="6" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C155" s="5">
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="E155" s="5" t="s">
         <v>8</v>
@@ -15502,24 +15507,24 @@
         <v>9</v>
       </c>
       <c r="G155" s="6" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="H155" s="3" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="5" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C156" s="5">
         <v>2</v>
       </c>
       <c r="D156" s="5" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="E156" s="5" t="s">
         <v>8</v>
@@ -15528,24 +15533,24 @@
         <v>9</v>
       </c>
       <c r="G156" s="6" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="H156" s="3" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A157" s="5" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C157" s="5">
         <v>1</v>
       </c>
       <c r="D157" s="5" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
       <c r="E157" s="5" t="s">
         <v>8</v>
@@ -15554,10 +15559,10 @@
         <v>9</v>
       </c>
       <c r="G157" s="6" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed two rows from XLSX overriding the words incorrectly.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA3218A-17B6-4A17-B082-A5ABE5F945C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFBED7EC-649E-4B35-9E81-2E46F075B0ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2180" yWindow="1920" windowWidth="19180" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="499">
   <si>
     <t>interview</t>
   </si>
@@ -2556,24 +2556,6 @@
   </si>
   <si>
     <t>f061280ca0edb626b22688f3a7d62420</t>
-  </si>
-  <si>
-    <t>0557fa923dcee4d0f86b1409f5c2167f</t>
-  </si>
-  <si>
-    <t>Back</t>
-  </si>
-  <si>
-    <t>Atrás</t>
-  </si>
-  <si>
-    <t>10ac3d04253ef7e1ddc73e6091c0cd55</t>
-  </si>
-  <si>
-    <t>Next</t>
-  </si>
-  <si>
-    <t>Siguiente</t>
   </si>
   <si>
     <t>Block_22</t>
@@ -11478,7 +11460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H155"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="57.453125" customWidth="1"/>
@@ -11517,7 +11499,7 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>289</v>
@@ -11535,15 +11517,15 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>289</v>
@@ -11561,24 +11543,24 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>289</v>
       </c>
       <c r="C4" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>292</v>
+        <v>462</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11587,24 +11569,24 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>294</v>
+        <v>463</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>485</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>289</v>
       </c>
       <c r="C5" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>295</v>
+        <v>366</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>8</v>
@@ -11613,24 +11595,24 @@
         <v>9</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>297</v>
+        <v>367</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>484</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>289</v>
+        <v>14</v>
       </c>
       <c r="C6" s="5">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>468</v>
+        <v>15</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>8</v>
@@ -11639,24 +11621,24 @@
         <v>9</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>469</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>491</v>
+        <v>16</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>289</v>
+        <v>14</v>
       </c>
       <c r="C7" s="5">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>372</v>
+        <v>17</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11665,24 +11647,24 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>490</v>
+        <v>368</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>8</v>
@@ -11691,24 +11673,24 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>8</v>
@@ -11717,24 +11699,24 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>374</v>
+        <v>54</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>8</v>
@@ -11743,24 +11725,24 @@
         <v>9</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>19</v>
+        <v>369</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>8</v>
@@ -11769,24 +11751,24 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>362</v>
+        <v>483</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="5">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>8</v>
@@ -11795,24 +11777,24 @@
         <v>9</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>375</v>
+        <v>24</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>8</v>
@@ -11821,24 +11803,24 @@
         <v>9</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>58</v>
+        <v>357</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="5">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>8</v>
@@ -11847,24 +11829,24 @@
         <v>9</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="5">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>8</v>
@@ -11873,24 +11855,24 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>8</v>
@@ -11899,24 +11881,24 @@
         <v>9</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C17" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>8</v>
@@ -11925,24 +11907,24 @@
         <v>9</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="5">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>8</v>
@@ -11951,24 +11933,24 @@
         <v>9</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="5">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>8</v>
@@ -11977,24 +11959,24 @@
         <v>9</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C20" s="5">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>8</v>
@@ -12003,24 +11985,24 @@
         <v>9</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C21" s="5">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>8</v>
@@ -12029,24 +12011,24 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>366</v>
+        <v>38</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>484</v>
+        <v>229</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="5">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>8</v>
@@ -12055,24 +12037,24 @@
         <v>9</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="5">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>8</v>
@@ -12081,24 +12063,24 @@
         <v>9</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>229</v>
+        <v>477</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="5">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>8</v>
@@ -12107,24 +12089,24 @@
         <v>9</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>230</v>
+        <v>480</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C25" s="5">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>8</v>
@@ -12133,24 +12115,24 @@
         <v>9</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>483</v>
+        <v>231</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="5">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>8</v>
@@ -12159,24 +12141,24 @@
         <v>9</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>486</v>
+        <v>232</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C27" s="5">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>8</v>
@@ -12185,24 +12167,24 @@
         <v>9</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C28" s="5">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>8</v>
@@ -12211,24 +12193,24 @@
         <v>9</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="5">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>8</v>
@@ -12237,24 +12219,24 @@
         <v>9</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>233</v>
+        <v>361</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="5">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>8</v>
@@ -12263,24 +12245,24 @@
         <v>9</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="5">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>8</v>
@@ -12289,24 +12271,24 @@
         <v>9</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>367</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="5">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>8</v>
@@ -12315,24 +12297,24 @@
         <v>9</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>235</v>
+        <v>476</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C33" s="5">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>8</v>
@@ -12341,24 +12323,24 @@
         <v>9</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C34" s="5">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>8</v>
@@ -12367,24 +12349,24 @@
         <v>9</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>482</v>
+        <v>238</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C35" s="5">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>8</v>
@@ -12393,24 +12375,24 @@
         <v>9</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="5">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E36" s="5" t="s">
         <v>8</v>
@@ -12419,24 +12401,24 @@
         <v>9</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C37" s="5">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E37" s="5" t="s">
         <v>8</v>
@@ -12445,24 +12427,24 @@
         <v>9</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C38" s="5">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>8</v>
@@ -12471,24 +12453,24 @@
         <v>9</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C39" s="5">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E39" s="5" t="s">
         <v>8</v>
@@ -12497,24 +12479,24 @@
         <v>9</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C40" s="5">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>8</v>
@@ -12523,24 +12505,24 @@
         <v>9</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="5">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>8</v>
@@ -12549,24 +12531,24 @@
         <v>9</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C42" s="5">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E42" s="5" t="s">
         <v>8</v>
@@ -12575,24 +12557,24 @@
         <v>9</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C43" s="5">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E43" s="5" t="s">
         <v>8</v>
@@ -12601,24 +12583,24 @@
         <v>9</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>245</v>
+        <v>475</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="5">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E44" s="5" t="s">
         <v>8</v>
@@ -12627,24 +12609,24 @@
         <v>9</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C45" s="5">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>8</v>
@@ -12653,24 +12635,24 @@
         <v>9</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>481</v>
+        <v>248</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C46" s="5">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>8</v>
@@ -12679,24 +12661,24 @@
         <v>9</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C47" s="5">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>8</v>
@@ -12705,24 +12687,24 @@
         <v>9</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>248</v>
+        <v>473</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C48" s="5">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>8</v>
@@ -12731,24 +12713,24 @@
         <v>9</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C49" s="5">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>8</v>
@@ -12757,24 +12739,24 @@
         <v>9</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C50" s="5">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E50" s="5" t="s">
         <v>8</v>
@@ -12783,24 +12765,24 @@
         <v>9</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C51" s="5">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>8</v>
@@ -12809,24 +12791,24 @@
         <v>9</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>480</v>
+        <v>252</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C52" s="5">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E52" s="5" t="s">
         <v>8</v>
@@ -12835,24 +12817,24 @@
         <v>9</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C53" s="5">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="E53" s="5" t="s">
         <v>8</v>
@@ -12861,24 +12843,24 @@
         <v>9</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C54" s="5">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E54" s="5" t="s">
         <v>8</v>
@@ -12887,24 +12869,24 @@
         <v>9</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C55" s="5">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>8</v>
@@ -12913,24 +12895,24 @@
         <v>9</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>14</v>
+        <v>107</v>
       </c>
       <c r="C56" s="5">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>8</v>
@@ -12939,24 +12921,24 @@
         <v>9</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="C57" s="5">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>8</v>
@@ -12965,24 +12947,24 @@
         <v>9</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C58" s="5">
         <v>0</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>8</v>
@@ -12991,24 +12973,24 @@
         <v>9</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C59" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E59" s="5" t="s">
         <v>8</v>
@@ -13017,24 +12999,24 @@
         <v>9</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>258</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>113</v>
       </c>
       <c r="C60" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>8</v>
@@ -13043,24 +13025,24 @@
         <v>9</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>113</v>
       </c>
       <c r="C61" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>8</v>
@@ -13069,24 +13051,24 @@
         <v>9</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>13</v>
+        <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>113</v>
       </c>
       <c r="C62" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>8</v>
@@ -13095,24 +13077,24 @@
         <v>9</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>113</v>
       </c>
       <c r="C63" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>8</v>
@@ -13121,24 +13103,24 @@
         <v>9</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>121</v>
+        <v>262</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>113</v>
+        <v>12</v>
       </c>
       <c r="C64" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>8</v>
@@ -13147,24 +13129,24 @@
         <v>9</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>113</v>
+        <v>12</v>
       </c>
       <c r="C65" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>8</v>
@@ -13173,24 +13155,24 @@
         <v>9</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>262</v>
+        <v>129</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>264</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C66" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E66" s="5" t="s">
         <v>8</v>
@@ -13199,24 +13181,24 @@
         <v>9</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C67" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>8</v>
@@ -13225,24 +13207,24 @@
         <v>9</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H67" s="4" t="s">
-        <v>264</v>
+        <v>133</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>266</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C68" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E68" s="5" t="s">
         <v>8</v>
@@ -13251,24 +13233,24 @@
         <v>9</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C69" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E69" s="5" t="s">
         <v>8</v>
@@ -13277,24 +13259,24 @@
         <v>9</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="C70" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E70" s="5" t="s">
         <v>8</v>
@@ -13303,24 +13285,24 @@
         <v>9</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="C71" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E71" s="5" t="s">
         <v>8</v>
@@ -13329,24 +13311,24 @@
         <v>9</v>
       </c>
       <c r="G71" s="6" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C72" s="5">
         <v>0</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>8</v>
@@ -13355,24 +13337,24 @@
         <v>9</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>269</v>
+        <v>446</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C73" s="5">
         <v>1</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>8</v>
@@ -13381,24 +13363,24 @@
         <v>9</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>270</v>
+        <v>147</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>271</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>143</v>
+        <v>10</v>
       </c>
       <c r="C74" s="5">
         <v>0</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>8</v>
@@ -13407,24 +13389,24 @@
         <v>9</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="H74" s="3" t="s">
-        <v>452</v>
+        <v>149</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>445</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C75" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>8</v>
@@ -13433,24 +13415,24 @@
         <v>9</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="174" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="C76" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>8</v>
@@ -13459,24 +13441,24 @@
         <v>9</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>451</v>
+        <v>273</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C77" s="5">
         <v>0</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>8</v>
@@ -13485,24 +13467,24 @@
         <v>9</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C78" s="5">
         <v>1</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E78" s="5" t="s">
         <v>8</v>
@@ -13511,24 +13493,24 @@
         <v>9</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="H78" s="2" t="s">
-        <v>273</v>
+        <v>159</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>468</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C79" s="5">
         <v>0</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>8</v>
@@ -13537,24 +13519,24 @@
         <v>9</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="H79" s="2" t="s">
-        <v>274</v>
+        <v>162</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>275</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C80" s="5">
         <v>1</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>8</v>
@@ -13563,24 +13545,24 @@
         <v>9</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="H80" s="3" t="s">
-        <v>474</v>
+        <v>164</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>276</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>160</v>
       </c>
       <c r="C81" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E81" s="5" t="s">
         <v>8</v>
@@ -13589,24 +13571,24 @@
         <v>9</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="H81" s="3" t="s">
-        <v>275</v>
+        <v>166</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>496</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>160</v>
       </c>
       <c r="C82" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E82" s="5" t="s">
         <v>8</v>
@@ -13615,24 +13597,24 @@
         <v>9</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="H82" s="2" t="s">
-        <v>276</v>
+        <v>168</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>277</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>160</v>
       </c>
       <c r="C83" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E83" s="5" t="s">
         <v>8</v>
@@ -13641,24 +13623,24 @@
         <v>9</v>
       </c>
       <c r="G83" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="H83" s="2" t="s">
-        <v>502</v>
+        <v>170</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>486</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C84" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E84" s="5" t="s">
         <v>8</v>
@@ -13667,24 +13649,24 @@
         <v>9</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="H84" s="3" t="s">
-        <v>277</v>
+        <v>173</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C85" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>8</v>
@@ -13693,24 +13675,24 @@
         <v>9</v>
       </c>
       <c r="G85" s="6" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>492</v>
+        <v>469</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>171</v>
+        <v>11</v>
       </c>
       <c r="C86" s="5">
         <v>0</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E86" s="5" t="s">
         <v>8</v>
@@ -13719,24 +13701,24 @@
         <v>9</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>173</v>
+        <v>372</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>171</v>
+        <v>11</v>
       </c>
       <c r="C87" s="5">
         <v>1</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>8</v>
@@ -13745,24 +13727,24 @@
         <v>9</v>
       </c>
       <c r="G87" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>475</v>
+        <v>278</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="C88" s="5">
         <v>0</v>
       </c>
       <c r="D88" s="5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>8</v>
@@ -13771,24 +13753,24 @@
         <v>9</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>378</v>
+        <v>181</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>503</v>
+        <v>279</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="C89" s="5">
         <v>1</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>8</v>
@@ -13797,24 +13779,24 @@
         <v>9</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>278</v>
+        <v>470</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C90" s="5">
         <v>0</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>8</v>
@@ -13823,24 +13805,24 @@
         <v>9</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="H90" s="2" t="s">
-        <v>279</v>
+        <v>186</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>280</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C91" s="5">
         <v>1</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>8</v>
@@ -13849,24 +13831,24 @@
         <v>9</v>
       </c>
       <c r="G91" s="6" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>476</v>
+        <v>281</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C92" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E92" s="5" t="s">
         <v>8</v>
@@ -13875,24 +13857,24 @@
         <v>9</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C93" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E93" s="5" t="s">
         <v>8</v>
@@ -13901,24 +13883,24 @@
         <v>9</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="H93" s="3" t="s">
-        <v>281</v>
+        <v>192</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C94" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>8</v>
@@ -13927,24 +13909,24 @@
         <v>9</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C95" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>8</v>
@@ -13953,24 +13935,24 @@
         <v>9</v>
       </c>
       <c r="G95" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="H95" s="2" t="s">
-        <v>283</v>
+        <v>196</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C96" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>8</v>
@@ -13979,24 +13961,24 @@
         <v>9</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C97" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>8</v>
@@ -14005,24 +13987,24 @@
         <v>9</v>
       </c>
       <c r="G97" s="6" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C98" s="5">
         <v>0</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>8</v>
@@ -14031,24 +14013,24 @@
         <v>9</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>199</v>
+        <v>489</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>286</v>
+        <v>488</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C99" s="5">
         <v>1</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>8</v>
@@ -14057,24 +14039,24 @@
         <v>9</v>
       </c>
       <c r="G99" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="H99" s="3" t="s">
-        <v>287</v>
+        <v>355</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>288</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C100" s="5">
         <v>0</v>
       </c>
       <c r="D100" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E100" s="5" t="s">
         <v>8</v>
@@ -14083,24 +14065,24 @@
         <v>9</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C101" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>8</v>
@@ -14109,24 +14091,24 @@
         <v>9</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>361</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>288</v>
+        <v>494</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C102" s="5">
         <v>0</v>
       </c>
       <c r="D102" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E102" s="5" t="s">
         <v>8</v>
@@ -14135,24 +14117,24 @@
         <v>9</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>499</v>
+        <v>261</v>
       </c>
     </row>
-    <row r="103" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E103" s="5" t="s">
         <v>8</v>
@@ -14161,24 +14143,24 @@
         <v>9</v>
       </c>
       <c r="G103" s="6" t="s">
-        <v>500</v>
+        <v>363</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>260</v>
+        <v>364</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C104" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>8</v>
@@ -14187,24 +14169,24 @@
         <v>9</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>501</v>
+        <v>214</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>261</v>
+        <v>365</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C105" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>8</v>
@@ -14213,24 +14195,24 @@
         <v>9</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="H105" s="3" t="s">
-        <v>370</v>
+        <v>217</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>351</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C106" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E106" s="5" t="s">
         <v>8</v>
@@ -14239,24 +14221,24 @@
         <v>9</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>371</v>
+        <v>350</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C107" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>216</v>
+        <v>353</v>
       </c>
       <c r="E107" s="5" t="s">
         <v>8</v>
@@ -14265,24 +14247,24 @@
         <v>9</v>
       </c>
       <c r="G107" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="H107" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>376</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>218</v>
+        <v>292</v>
       </c>
       <c r="C108" s="5">
         <v>0</v>
       </c>
       <c r="D108" s="5" t="s">
-        <v>219</v>
+        <v>378</v>
       </c>
       <c r="E108" s="5" t="s">
         <v>8</v>
@@ -14291,24 +14273,24 @@
         <v>9</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="H108" s="3" t="s">
-        <v>356</v>
+        <v>379</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>382</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>218</v>
+        <v>292</v>
       </c>
       <c r="C109" s="5">
         <v>1</v>
       </c>
       <c r="D109" s="5" t="s">
-        <v>359</v>
+        <v>380</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>8</v>
@@ -14317,24 +14299,24 @@
         <v>9</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="H109" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
+      </c>
+      <c r="H109" s="2" t="s">
+        <v>383</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C110" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D110" s="5" t="s">
-        <v>384</v>
+        <v>293</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>8</v>
@@ -14343,24 +14325,24 @@
         <v>9</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>385</v>
+        <v>294</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>388</v>
+        <v>352</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C111" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>386</v>
+        <v>296</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>8</v>
@@ -14369,21 +14351,21 @@
         <v>9</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="H111" s="2" t="s">
-        <v>389</v>
+        <v>297</v>
+      </c>
+      <c r="H111" s="3" t="s">
+        <v>298</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C112" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>299</v>
@@ -14397,22 +14379,22 @@
       <c r="G112" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="H112" s="2" t="s">
-        <v>358</v>
+      <c r="H112" s="3" t="s">
+        <v>384</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B113" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C113" s="5">
+        <v>2</v>
+      </c>
+      <c r="D113" s="5" t="s">
         <v>301</v>
-      </c>
-      <c r="C113" s="5">
-        <v>0</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>302</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>8</v>
@@ -14421,24 +14403,24 @@
         <v>9</v>
       </c>
       <c r="G113" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A114" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C114" s="5">
+        <v>3</v>
+      </c>
+      <c r="D114" s="5" t="s">
         <v>303</v>
-      </c>
-      <c r="H113" s="3" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C114" s="5">
-        <v>1</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>305</v>
       </c>
       <c r="E114" s="5" t="s">
         <v>8</v>
@@ -14447,24 +14429,24 @@
         <v>9</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C115" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D115" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E115" s="5" t="s">
         <v>8</v>
@@ -14473,24 +14455,24 @@
         <v>9</v>
       </c>
       <c r="G115" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="H115" s="2" t="s">
-        <v>391</v>
+        <v>306</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C116" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D116" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E116" s="5" t="s">
         <v>8</v>
@@ -14499,21 +14481,21 @@
         <v>9</v>
       </c>
       <c r="G116" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="H116" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="H116" s="3" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C117" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>311</v>
@@ -14527,19 +14509,19 @@
       <c r="G117" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="H117" s="3" t="s">
+      <c r="H117" s="2" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C118" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>314</v>
@@ -14553,22 +14535,22 @@
       <c r="G118" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="H118" s="3" t="s">
+      <c r="H118" s="2" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="C119" s="5">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>8</v>
@@ -14577,24 +14559,24 @@
         <v>9</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H119" s="2" t="s">
-        <v>319</v>
+        <v>387</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="C120" s="5">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>8</v>
@@ -14603,18 +14585,18 @@
         <v>9</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>321</v>
-      </c>
-      <c r="H120" s="2" t="s">
         <v>322</v>
       </c>
+      <c r="H120" s="3" t="s">
+        <v>323</v>
+      </c>
     </row>
-    <row r="121" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>323</v>
+        <v>11</v>
       </c>
       <c r="C121" s="5">
         <v>0</v>
@@ -14632,21 +14614,21 @@
         <v>325</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>393</v>
+        <v>326</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>326</v>
+        <v>11</v>
       </c>
       <c r="C122" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>327</v>
+        <v>490</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>8</v>
@@ -14655,24 +14637,24 @@
         <v>9</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="H122" s="3" t="s">
-        <v>329</v>
+        <v>491</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>498</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C123" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D123" s="5" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>8</v>
@@ -14681,24 +14663,24 @@
         <v>9</v>
       </c>
       <c r="G123" s="6" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="H123" s="2" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C124" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>496</v>
+        <v>177</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>8</v>
@@ -14707,24 +14689,24 @@
         <v>9</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>497</v>
-      </c>
-      <c r="H124" s="2" t="s">
-        <v>504</v>
+        <v>178</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>278</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>11</v>
+        <v>394</v>
       </c>
       <c r="C125" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>333</v>
+        <v>395</v>
       </c>
       <c r="E125" s="5" t="s">
         <v>8</v>
@@ -14733,24 +14715,24 @@
         <v>9</v>
       </c>
       <c r="G125" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>335</v>
+        <v>396</v>
+      </c>
+      <c r="H125" s="8" t="s">
+        <v>458</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>11</v>
+        <v>394</v>
       </c>
       <c r="C126" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>177</v>
+        <v>397</v>
       </c>
       <c r="E126" s="5" t="s">
         <v>8</v>
@@ -14759,24 +14741,24 @@
         <v>9</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="H126" s="3" t="s">
-        <v>278</v>
+        <v>398</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>455</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="C127" s="5">
+        <v>2</v>
+      </c>
+      <c r="D127" s="5" t="s">
         <v>399</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="C127" s="5">
-        <v>0</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>401</v>
       </c>
       <c r="E127" s="5" t="s">
         <v>8</v>
@@ -14785,24 +14767,24 @@
         <v>9</v>
       </c>
       <c r="G127" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="H127" s="8" t="s">
-        <v>464</v>
+        <v>400</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>457</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>400</v>
+        <v>335</v>
       </c>
       <c r="C128" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E128" s="5" t="s">
         <v>8</v>
@@ -14811,24 +14793,22 @@
         <v>9</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>461</v>
-      </c>
+        <v>402</v>
+      </c>
+      <c r="H128" s="7"/>
     </row>
-    <row r="129" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>400</v>
+        <v>335</v>
       </c>
       <c r="C129" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E129" s="5" t="s">
         <v>8</v>
@@ -14837,24 +14817,24 @@
         <v>9</v>
       </c>
       <c r="G129" s="6" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C130" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E130" s="5" t="s">
         <v>8</v>
@@ -14863,22 +14843,24 @@
         <v>9</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="H130" s="7"/>
+        <v>406</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>471</v>
+      </c>
     </row>
-    <row r="131" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C131" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D131" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>8</v>
@@ -14887,24 +14869,24 @@
         <v>9</v>
       </c>
       <c r="G131" s="6" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="H131" s="2" t="s">
-        <v>459</v>
+        <v>472</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>341</v>
+        <v>171</v>
       </c>
       <c r="C132" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E132" s="5" t="s">
         <v>8</v>
@@ -14913,24 +14895,22 @@
         <v>9</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="H132" s="2" t="s">
-        <v>477</v>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="H132" s="7"/>
     </row>
-    <row r="133" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>341</v>
+        <v>171</v>
       </c>
       <c r="C133" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>8</v>
@@ -14939,24 +14919,24 @@
         <v>9</v>
       </c>
       <c r="G133" s="6" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>478</v>
+        <v>454</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C134" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E134" s="5" t="s">
         <v>8</v>
@@ -14965,22 +14945,24 @@
         <v>9</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="H134" s="7"/>
+        <v>414</v>
+      </c>
+      <c r="H134" s="2" t="s">
+        <v>444</v>
+      </c>
     </row>
-    <row r="135" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C135" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>8</v>
@@ -14989,24 +14971,24 @@
         <v>9</v>
       </c>
       <c r="G135" s="6" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="H135" s="2" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
     </row>
-    <row r="136" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C136" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>8</v>
@@ -15015,24 +14997,24 @@
         <v>9</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>171</v>
+        <v>419</v>
       </c>
       <c r="C137" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>8</v>
@@ -15041,24 +15023,22 @@
         <v>9</v>
       </c>
       <c r="G137" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="H137" s="7"/>
+    </row>
+    <row r="138" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+      <c r="A138" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="C138" s="5">
+        <v>1</v>
+      </c>
+      <c r="D138" s="5" t="s">
         <v>422</v>
-      </c>
-      <c r="H137" s="2" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A138" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C138" s="5">
-        <v>4</v>
-      </c>
-      <c r="D138" s="5" t="s">
-        <v>423</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>8</v>
@@ -15067,24 +15047,24 @@
         <v>9</v>
       </c>
       <c r="G138" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="H138" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A139" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="C139" s="5">
+        <v>2</v>
+      </c>
+      <c r="D139" s="5" t="s">
         <v>424</v>
-      </c>
-      <c r="H138" s="2" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A139" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B139" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="C139" s="5">
-        <v>0</v>
-      </c>
-      <c r="D139" s="5" t="s">
-        <v>426</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>8</v>
@@ -15093,22 +15073,24 @@
         <v>9</v>
       </c>
       <c r="G139" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="H139" s="2" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A140" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="C140" s="5">
+        <v>0</v>
+      </c>
+      <c r="D140" s="5" t="s">
         <v>427</v>
-      </c>
-      <c r="H139" s="7"/>
-    </row>
-    <row r="140" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A140" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B140" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="C140" s="5">
-        <v>1</v>
-      </c>
-      <c r="D140" s="5" t="s">
-        <v>428</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>8</v>
@@ -15117,24 +15099,24 @@
         <v>9</v>
       </c>
       <c r="G140" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="H140" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A141" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="C141" s="5">
+        <v>1</v>
+      </c>
+      <c r="D141" s="5" t="s">
         <v>429</v>
-      </c>
-      <c r="H140" s="2" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="A141" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B141" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="C141" s="5">
-        <v>2</v>
-      </c>
-      <c r="D141" s="5" t="s">
-        <v>430</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>8</v>
@@ -15143,24 +15125,24 @@
         <v>9</v>
       </c>
       <c r="G141" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="H141" s="2" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A142" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="C142" s="5">
+        <v>2</v>
+      </c>
+      <c r="D142" s="5" t="s">
         <v>431</v>
-      </c>
-      <c r="H141" s="2" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A142" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="C142" s="5">
-        <v>0</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>433</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>8</v>
@@ -15169,24 +15151,24 @@
         <v>9</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>432</v>
+        <v>340</v>
       </c>
       <c r="C143" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D143" s="5" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>8</v>
@@ -15195,24 +15177,24 @@
         <v>9</v>
       </c>
       <c r="G143" s="6" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H143" s="2" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>432</v>
+        <v>340</v>
       </c>
       <c r="C144" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="E144" s="5" t="s">
         <v>8</v>
@@ -15221,24 +15203,24 @@
         <v>9</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="C145" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>8</v>
@@ -15247,24 +15229,24 @@
         <v>9</v>
       </c>
       <c r="G145" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="H145" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A146" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="B146" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="C146" s="5">
+        <v>0</v>
+      </c>
+      <c r="D146" s="5" t="s">
         <v>440</v>
-      </c>
-      <c r="H145" s="2" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A146" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="B146" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C146" s="5">
-        <v>1</v>
-      </c>
-      <c r="D146" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>8</v>
@@ -15273,24 +15255,24 @@
         <v>9</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>454</v>
+        <v>441</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A147" s="5" t="s">
-        <v>399</v>
+        <v>330</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="C147" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>443</v>
+        <v>391</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>8</v>
@@ -15299,24 +15281,24 @@
         <v>9</v>
       </c>
       <c r="G147" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="H147" s="2" t="s">
-        <v>453</v>
+        <v>392</v>
+      </c>
+      <c r="H147" s="3" t="s">
+        <v>332</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>336</v>
+        <v>375</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>445</v>
+        <v>331</v>
       </c>
       <c r="C148" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>446</v>
+        <v>333</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>8</v>
@@ -15325,24 +15307,24 @@
         <v>9</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>447</v>
+        <v>334</v>
       </c>
       <c r="H148" s="2" t="s">
-        <v>447</v>
+        <v>388</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
-        <v>336</v>
+        <v>375</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C149" s="5">
         <v>0</v>
       </c>
       <c r="D149" s="5" t="s">
-        <v>397</v>
+        <v>336</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>8</v>
@@ -15351,24 +15333,24 @@
         <v>9</v>
       </c>
       <c r="G149" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="H149" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>377</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A150" s="5" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C150" s="5">
         <v>1</v>
       </c>
       <c r="D150" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>8</v>
@@ -15377,24 +15359,24 @@
         <v>9</v>
       </c>
       <c r="G150" s="6" t="s">
-        <v>340</v>
+        <v>389</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>394</v>
+        <v>464</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A151" s="5" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C151" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E151" s="5" t="s">
         <v>8</v>
@@ -15403,24 +15385,24 @@
         <v>9</v>
       </c>
       <c r="G151" s="6" t="s">
-        <v>343</v>
+        <v>460</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>383</v>
+        <v>461</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A152" s="5" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="B152" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="C152" s="5">
+        <v>0</v>
+      </c>
+      <c r="D152" s="5" t="s">
         <v>341</v>
-      </c>
-      <c r="C152" s="5">
-        <v>1</v>
-      </c>
-      <c r="D152" s="5" t="s">
-        <v>344</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>8</v>
@@ -15429,24 +15411,24 @@
         <v>9</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>395</v>
+        <v>342</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>470</v>
+        <v>343</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A153" s="5" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C153" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E153" s="5" t="s">
         <v>8</v>
@@ -15455,21 +15437,21 @@
         <v>9</v>
       </c>
       <c r="G153" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="H153" s="2" t="s">
-        <v>467</v>
+        <v>345</v>
+      </c>
+      <c r="H153" s="3" t="s">
+        <v>346</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="C154" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D154" s="5" t="s">
         <v>347</v>
@@ -15483,22 +15465,22 @@
       <c r="G154" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="H154" s="2" t="s">
+      <c r="H154" s="3" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>346</v>
+        <v>215</v>
       </c>
       <c r="C155" s="5">
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
-        <v>350</v>
+        <v>465</v>
       </c>
       <c r="E155" s="5" t="s">
         <v>8</v>
@@ -15507,62 +15489,10 @@
         <v>9</v>
       </c>
       <c r="G155" s="6" t="s">
-        <v>351</v>
-      </c>
-      <c r="H155" s="3" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A156" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="B156" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C156" s="5">
-        <v>2</v>
-      </c>
-      <c r="D156" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="E156" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F156" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G156" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="H156" s="3" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A157" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="B157" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="C157" s="5">
-        <v>1</v>
-      </c>
-      <c r="D157" s="5" t="s">
-        <v>471</v>
-      </c>
-      <c r="E157" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G157" s="6" t="s">
-        <v>472</v>
-      </c>
-      <c r="H157" s="2" t="s">
-        <v>473</v>
+        <v>466</v>
+      </c>
+      <c r="H155" s="2" t="s">
+        <v>467</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replaced defaulted AL words for custom ILAO words.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D525B93-099F-464D-880D-D1F57E1FB6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2031E34-7659-4F9B-B844-4F598EF64059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6120" yWindow="2090" windowWidth="25060" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5260" yWindow="2750" windowWidth="25060" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="508">
   <si>
     <t>interview</t>
   </si>
@@ -2522,31 +2522,6 @@
   </si>
   <si>
     <t>**PLACEHOLDER - ¿Qué significa firmar los formularios?**</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Después de hacer clic en **Siguiente**, puede tomar unos momentos para terminar de hacer tus formularios.
-###### No necesitas actualizar tu pantalla. ¡Ánimo!
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[NEWLINE]</t>
-    </r>
   </si>
   <si>
     <t>Block_3</t>
@@ -11064,6 +11039,43 @@
   </si>
   <si>
     <t>Continuar</t>
+  </si>
+  <si>
+    <t>docassemble.AssemblyLine:data/questions/al_visual.yml</t>
+  </si>
+  <si>
+    <t>b7ee3531c0640e07d45978804005b1a6</t>
+  </si>
+  <si>
+    <t>Atrás</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Después de hacer clic en **Continuar**, puede tomar unos momentos para terminar de hacer tus formularios.
+###### No necesitas actualizar tu pantalla. ¡Ánimo!
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[NEWLINE]</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -11475,7 +11487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="57.453125" customWidth="1"/>
@@ -11514,16 +11526,16 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>8</v>
@@ -11532,24 +11544,24 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>8</v>
@@ -11558,93 +11570,93 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C4" s="5">
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>461</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C5" s="5">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>366</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>14</v>
@@ -11670,7 +11682,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
@@ -11688,15 +11700,15 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
@@ -11722,7 +11734,7 @@
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
@@ -11743,12 +11755,12 @@
         <v>54</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>14</v>
@@ -11766,7 +11778,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>223</v>
@@ -11774,7 +11786,7 @@
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>14</v>
@@ -11795,12 +11807,12 @@
         <v>58</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>14</v>
@@ -11826,7 +11838,7 @@
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -11844,15 +11856,15 @@
         <v>9</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11878,7 +11890,7 @@
     </row>
     <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11896,15 +11908,15 @@
         <v>9</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11930,7 +11942,7 @@
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11948,15 +11960,15 @@
         <v>9</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -11982,7 +11994,7 @@
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -12000,15 +12012,15 @@
         <v>9</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -12034,7 +12046,7 @@
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -12060,7 +12072,7 @@
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -12086,7 +12098,7 @@
     </row>
     <row r="24" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -12107,12 +12119,12 @@
         <v>42</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -12133,12 +12145,12 @@
         <v>44</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -12164,7 +12176,7 @@
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -12190,7 +12202,7 @@
     </row>
     <row r="28" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -12216,7 +12228,7 @@
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -12242,7 +12254,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -12263,12 +12275,12 @@
         <v>54</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -12294,7 +12306,7 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -12320,7 +12332,7 @@
     </row>
     <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -12341,12 +12353,12 @@
         <v>60</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -12372,7 +12384,7 @@
     </row>
     <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -12398,7 +12410,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -12424,7 +12436,7 @@
     </row>
     <row r="37" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12450,7 +12462,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12476,7 +12488,7 @@
     </row>
     <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12502,7 +12514,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12528,7 +12540,7 @@
     </row>
     <row r="41" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12554,7 +12566,7 @@
     </row>
     <row r="42" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12580,7 +12592,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12606,7 +12618,7 @@
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12627,12 +12639,12 @@
         <v>82</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12658,7 +12670,7 @@
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12684,7 +12696,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12710,7 +12722,7 @@
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12731,12 +12743,12 @@
         <v>90</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12762,7 +12774,7 @@
     </row>
     <row r="50" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -12783,12 +12795,12 @@
         <v>94</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -12814,7 +12826,7 @@
     </row>
     <row r="52" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -12840,7 +12852,7 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -12866,7 +12878,7 @@
     </row>
     <row r="54" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -12892,7 +12904,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -12918,7 +12930,7 @@
     </row>
     <row r="56" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -12944,7 +12956,7 @@
     </row>
     <row r="57" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>107</v>
@@ -12970,7 +12982,7 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>107</v>
@@ -12979,24 +12991,24 @@
         <v>1</v>
       </c>
       <c r="D58" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G58" s="6" t="s">
         <v>497</v>
       </c>
-      <c r="E58" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G58" s="6" t="s">
+      <c r="H58" s="2" t="s">
         <v>498</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>110</v>
@@ -13022,7 +13034,7 @@
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>113</v>
@@ -13048,7 +13060,7 @@
     </row>
     <row r="61" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>113</v>
@@ -13074,7 +13086,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>113</v>
@@ -13100,7 +13112,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>113</v>
@@ -13126,7 +13138,7 @@
     </row>
     <row r="64" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>113</v>
@@ -13152,7 +13164,7 @@
     </row>
     <row r="65" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>113</v>
@@ -13178,7 +13190,7 @@
     </row>
     <row r="66" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>12</v>
@@ -13204,7 +13216,7 @@
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>12</v>
@@ -13230,7 +13242,7 @@
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>12</v>
@@ -13256,7 +13268,7 @@
     </row>
     <row r="69" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>12</v>
@@ -13282,7 +13294,7 @@
     </row>
     <row r="70" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>12</v>
@@ -13308,7 +13320,7 @@
     </row>
     <row r="71" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>12</v>
@@ -13334,7 +13346,7 @@
     </row>
     <row r="72" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>138</v>
@@ -13360,7 +13372,7 @@
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>138</v>
@@ -13386,7 +13398,7 @@
     </row>
     <row r="74" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>143</v>
@@ -13407,12 +13419,12 @@
         <v>145</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>143</v>
@@ -13438,7 +13450,7 @@
     </row>
     <row r="76" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>10</v>
@@ -13459,12 +13471,12 @@
         <v>149</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>150</v>
@@ -13490,7 +13502,7 @@
     </row>
     <row r="78" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>150</v>
@@ -13516,7 +13528,7 @@
     </row>
     <row r="79" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>155</v>
@@ -13542,7 +13554,7 @@
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>155</v>
@@ -13563,12 +13575,12 @@
         <v>159</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>160</v>
@@ -13594,7 +13606,7 @@
     </row>
     <row r="82" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>160</v>
@@ -13620,7 +13632,7 @@
     </row>
     <row r="83" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>160</v>
@@ -13641,12 +13653,12 @@
         <v>166</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>160</v>
@@ -13672,7 +13684,7 @@
     </row>
     <row r="85" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>160</v>
@@ -13693,12 +13705,12 @@
         <v>170</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>171</v>
@@ -13719,12 +13731,12 @@
         <v>173</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>171</v>
@@ -13745,12 +13757,12 @@
         <v>175</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>11</v>
@@ -13768,128 +13780,128 @@
         <v>9</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>370</v>
+        <v>503</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C89" s="5">
         <v>1</v>
       </c>
       <c r="D89" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F89" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A90" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C90" s="5">
+        <v>1</v>
+      </c>
+      <c r="D90" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E89" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F89" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G89" s="6" t="s">
+      <c r="E90" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G90" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="H89" s="3" t="s">
+      <c r="H90" s="3" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="A90" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C90" s="5">
-        <v>0</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F90" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G90" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="H90" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>179</v>
       </c>
       <c r="C91" s="5">
+        <v>0</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F91" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A92" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C92" s="5">
         <v>1</v>
       </c>
-      <c r="D91" s="5" t="s">
+      <c r="D92" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="E91" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G91" s="6" t="s">
+      <c r="E92" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G92" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="H91" s="3" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="C92" s="5">
-        <v>0</v>
-      </c>
-      <c r="D92" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F92" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G92" s="6" t="s">
-        <v>186</v>
-      </c>
       <c r="H92" s="3" t="s">
-        <v>280</v>
+        <v>467</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C93" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E93" s="5" t="s">
         <v>8</v>
@@ -13898,24 +13910,24 @@
         <v>9</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C94" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D94" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>8</v>
@@ -13924,24 +13936,24 @@
         <v>9</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C95" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>8</v>
@@ -13950,24 +13962,24 @@
         <v>9</v>
       </c>
       <c r="G95" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="H95" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C96" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D96" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>8</v>
@@ -13976,24 +13988,24 @@
         <v>9</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="H96" s="3" t="s">
-        <v>284</v>
+        <v>192</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C97" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>8</v>
@@ -14002,24 +14014,24 @@
         <v>9</v>
       </c>
       <c r="G97" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="C98" s="5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>8</v>
@@ -14028,103 +14040,103 @@
         <v>9</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>197</v>
       </c>
       <c r="C99" s="5">
+        <v>0</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F99" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G99" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A100" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C100" s="5">
         <v>1</v>
       </c>
-      <c r="D99" s="5" t="s">
+      <c r="D100" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="E99" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F99" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G99" s="6" t="s">
+      <c r="E100" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G100" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="H99" s="3" t="s">
+      <c r="H100" s="3" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A100" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="C100" s="5">
-        <v>0</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F100" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G100" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="H100" s="3" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>202</v>
       </c>
       <c r="C101" s="5">
+        <v>0</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G101" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+      <c r="A102" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C102" s="5">
         <v>1</v>
       </c>
-      <c r="D101" s="5" t="s">
+      <c r="D102" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="E101" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F101" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G101" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A102" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="C102" s="5">
-        <v>0</v>
-      </c>
-      <c r="D102" s="5" t="s">
-        <v>206</v>
-      </c>
       <c r="E102" s="5" t="s">
         <v>8</v>
       </c>
@@ -14132,24 +14144,24 @@
         <v>9</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="H102" s="3" t="s">
-        <v>491</v>
+        <v>353</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>507</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C103" s="5">
         <v>0</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E103" s="5" t="s">
         <v>8</v>
@@ -14158,24 +14170,24 @@
         <v>9</v>
       </c>
       <c r="G103" s="6" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>260</v>
+        <v>490</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C104" s="5">
         <v>0</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>8</v>
@@ -14184,24 +14196,24 @@
         <v>9</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C105" s="5">
         <v>0</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>8</v>
@@ -14210,76 +14222,76 @@
         <v>9</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>362</v>
+        <v>492</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>211</v>
       </c>
       <c r="C106" s="5">
+        <v>0</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E106" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G106" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A107" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C107" s="5">
         <v>1</v>
       </c>
-      <c r="D106" s="5" t="s">
+      <c r="D107" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="E106" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F106" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G106" s="6" t="s">
+      <c r="E107" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F107" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G107" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="H106" s="3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="107" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A107" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="C107" s="5">
-        <v>2</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E107" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F107" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G107" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="H107" s="2" t="s">
-        <v>350</v>
+      <c r="H107" s="3" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C108" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D108" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E108" s="5" t="s">
         <v>8</v>
@@ -14288,232 +14300,232 @@
         <v>9</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="H108" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="H108" s="2" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>218</v>
       </c>
       <c r="C109" s="5">
+        <v>0</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E109" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F109" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G109" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A110" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C110" s="5">
         <v>1</v>
       </c>
-      <c r="D109" s="5" t="s">
+      <c r="D110" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F110" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G110" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="E109" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F109" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G109" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="H109" s="3" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="110" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A110" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C110" s="5">
-        <v>0</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F110" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G110" s="6" t="s">
-        <v>378</v>
-      </c>
-      <c r="H110" s="2" t="s">
-        <v>381</v>
+      <c r="H110" s="3" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B111" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C111" s="5">
+        <v>0</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="E111" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F111" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G111" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="H111" s="2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C112" s="5">
+        <v>1</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="E112" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F112" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G112" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="H112" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A113" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="C113" s="5">
+        <v>2</v>
+      </c>
+      <c r="D113" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="C111" s="5">
+      <c r="E113" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F113" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G113" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A114" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C114" s="5">
+        <v>0</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F114" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G114" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A115" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C115" s="5">
         <v>1</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F111" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G111" s="6" t="s">
-        <v>380</v>
-      </c>
-      <c r="H111" s="2" t="s">
+      <c r="D115" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F115" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G115" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="H115" s="3" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A112" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="C112" s="5">
+    <row r="116" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A116" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C116" s="5">
         <v>2</v>
       </c>
-      <c r="D112" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="E112" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F112" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G112" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="H112" s="2" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A113" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C113" s="5">
-        <v>0</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="E113" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F113" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G113" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="H113" s="3" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C114" s="5">
-        <v>1</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="E114" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F114" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G114" s="6" t="s">
+      <c r="D116" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="H114" s="3" t="s">
+      <c r="E116" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F116" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G116" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="H116" s="2" t="s">
         <v>383</v>
-      </c>
-    </row>
-    <row r="115" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A115" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C115" s="5">
-        <v>2</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="E115" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F115" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G115" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="H115" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A116" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C116" s="5">
-        <v>3</v>
-      </c>
-      <c r="D116" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="E116" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F116" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G116" s="6" t="s">
-        <v>304</v>
-      </c>
-      <c r="H116" s="3" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C117" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E117" s="5" t="s">
         <v>8</v>
@@ -14522,24 +14534,24 @@
         <v>9</v>
       </c>
       <c r="G117" s="6" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>307</v>
+        <v>384</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C118" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>8</v>
@@ -14548,24 +14560,24 @@
         <v>9</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C119" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>8</v>
@@ -14574,76 +14586,76 @@
         <v>9</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="H119" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C120" s="5">
+        <v>6</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="H120" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A121" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C121" s="5">
         <v>7</v>
       </c>
-      <c r="D120" s="5" t="s">
+      <c r="D121" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G121" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="E120" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G120" s="6" t="s">
+      <c r="H121" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="H120" s="2" t="s">
+    </row>
+    <row r="122" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A122" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B122" s="5" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="121" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A121" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B121" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="C121" s="5">
-        <v>0</v>
-      </c>
-      <c r="D121" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="E121" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F121" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G121" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="H121" s="2" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="122" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A122" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>320</v>
       </c>
       <c r="C122" s="5">
         <v>0</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="E122" s="5" t="s">
         <v>8</v>
@@ -14652,24 +14664,24 @@
         <v>9</v>
       </c>
       <c r="G122" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="H122" s="3" t="s">
-        <v>323</v>
+        <v>318</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>385</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>11</v>
+        <v>319</v>
       </c>
       <c r="C123" s="5">
         <v>0</v>
       </c>
       <c r="D123" s="5" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>8</v>
@@ -14678,24 +14690,24 @@
         <v>9</v>
       </c>
       <c r="G123" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="124" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+      <c r="H123" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C124" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>488</v>
+        <v>323</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>8</v>
@@ -14704,24 +14716,24 @@
         <v>9</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>489</v>
+        <v>324</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C125" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>327</v>
+        <v>487</v>
       </c>
       <c r="E125" s="5" t="s">
         <v>8</v>
@@ -14730,254 +14742,256 @@
         <v>9</v>
       </c>
       <c r="G125" s="6" t="s">
-        <v>328</v>
+        <v>488</v>
       </c>
       <c r="H125" s="2" t="s">
-        <v>329</v>
+        <v>495</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C126" s="5">
+        <v>2</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F126" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G126" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A127" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C127" s="5">
         <v>3</v>
       </c>
-      <c r="D126" s="5" t="s">
+      <c r="D127" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="E126" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F126" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G126" s="6" t="s">
+      <c r="E127" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F127" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G127" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="H126" s="3" t="s">
+      <c r="H127" s="3" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A127" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B127" s="5" t="s">
+    <row r="128" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A128" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="C128" s="5">
+        <v>0</v>
+      </c>
+      <c r="D128" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="C127" s="5">
+      <c r="E128" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G128" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="H128" s="8" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+      <c r="A129" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="C129" s="5">
+        <v>1</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G129" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A130" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="C130" s="5">
+        <v>2</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G130" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A131" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C131" s="5">
         <v>0</v>
       </c>
-      <c r="D127" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G127" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="H127" s="8" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="128" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A128" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="C128" s="5">
+      <c r="D131" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G131" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="H131" s="7"/>
+    </row>
+    <row r="132" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A132" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C132" s="5">
         <v>1</v>
       </c>
-      <c r="D128" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="E128" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G128" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A129" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="C129" s="5">
+      <c r="D132" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G132" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A133" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C133" s="5">
         <v>2</v>
       </c>
-      <c r="D129" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="E129" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G129" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="H129" s="2" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A130" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C130" s="5">
-        <v>0</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="E130" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G130" s="6" t="s">
-        <v>400</v>
-      </c>
-      <c r="H130" s="7"/>
-    </row>
-    <row r="131" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A131" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C131" s="5">
-        <v>1</v>
-      </c>
-      <c r="D131" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="E131" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G131" s="6" t="s">
+      <c r="D133" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="H131" s="2" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="132" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A132" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C132" s="5">
-        <v>2</v>
-      </c>
-      <c r="D132" s="5" t="s">
+      <c r="E133" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F133" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G133" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="E132" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G132" s="6" t="s">
+      <c r="H133" s="2" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A134" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C134" s="5">
+        <v>3</v>
+      </c>
+      <c r="D134" s="5" t="s">
         <v>404</v>
       </c>
-      <c r="H132" s="2" t="s">
+      <c r="E134" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G134" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="H134" s="2" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A133" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B133" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C133" s="5">
-        <v>3</v>
-      </c>
-      <c r="D133" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="E133" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F133" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G133" s="6" t="s">
-        <v>406</v>
-      </c>
-      <c r="H133" s="2" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A134" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C134" s="5">
-        <v>0</v>
-      </c>
-      <c r="D134" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F134" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G134" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="H134" s="7"/>
-    </row>
-    <row r="135" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C135" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>8</v>
@@ -14986,24 +15000,22 @@
         <v>9</v>
       </c>
       <c r="G135" s="6" t="s">
-        <v>410</v>
-      </c>
-      <c r="H135" s="2" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>407</v>
+      </c>
+      <c r="H135" s="7"/>
+    </row>
+    <row r="136" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C136" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>8</v>
@@ -15012,24 +15024,24 @@
         <v>9</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C137" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>8</v>
@@ -15038,24 +15050,24 @@
         <v>9</v>
       </c>
       <c r="G137" s="6" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C138" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>8</v>
@@ -15064,127 +15076,127 @@
         <v>9</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B139" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C139" s="5">
+        <v>4</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G139" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="H139" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A140" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="C140" s="5">
+        <v>0</v>
+      </c>
+      <c r="D140" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="C139" s="5">
-        <v>0</v>
-      </c>
-      <c r="D139" s="5" t="s">
+      <c r="E140" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F140" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G140" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="E139" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G139" s="6" t="s">
+      <c r="H140" s="7"/>
+    </row>
+    <row r="141" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+      <c r="A141" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="C141" s="5">
+        <v>1</v>
+      </c>
+      <c r="D141" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="H139" s="7"/>
-    </row>
-    <row r="140" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A140" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B140" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="C140" s="5">
-        <v>1</v>
-      </c>
-      <c r="D140" s="5" t="s">
+      <c r="E141" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G141" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="E140" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G140" s="6" t="s">
+      <c r="H141" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A142" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="C142" s="5">
+        <v>2</v>
+      </c>
+      <c r="D142" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="H140" s="2" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="A141" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B141" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="C141" s="5">
-        <v>2</v>
-      </c>
-      <c r="D141" s="5" t="s">
+      <c r="E142" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G142" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="E141" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G141" s="6" t="s">
-        <v>423</v>
-      </c>
-      <c r="H141" s="2" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A142" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="C142" s="5">
-        <v>0</v>
-      </c>
-      <c r="D142" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="E142" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G142" s="6" t="s">
-        <v>426</v>
-      </c>
       <c r="H142" s="2" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B143" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="C143" s="5">
+        <v>0</v>
+      </c>
+      <c r="D143" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="C143" s="5">
-        <v>1</v>
-      </c>
-      <c r="D143" s="5" t="s">
-        <v>427</v>
-      </c>
       <c r="E143" s="5" t="s">
         <v>8</v>
       </c>
@@ -15192,24 +15204,24 @@
         <v>9</v>
       </c>
       <c r="G143" s="6" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="H143" s="2" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C144" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="E144" s="5" t="s">
         <v>8</v>
@@ -15218,24 +15230,24 @@
         <v>9</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="H144" s="2" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>339</v>
+        <v>423</v>
       </c>
       <c r="C145" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>8</v>
@@ -15244,7 +15256,7 @@
         <v>9</v>
       </c>
       <c r="G145" s="6" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="H145" s="2" t="s">
         <v>447</v>
@@ -15252,16 +15264,16 @@
     </row>
     <row r="146" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A146" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C146" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D146" s="5" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>8</v>
@@ -15270,24 +15282,24 @@
         <v>9</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="H146" s="2" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A147" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C147" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>8</v>
@@ -15296,24 +15308,24 @@
         <v>9</v>
       </c>
       <c r="G147" s="6" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="H147" s="2" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>437</v>
+        <v>338</v>
       </c>
       <c r="C148" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>8</v>
@@ -15322,244 +15334,270 @@
         <v>9</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="H148" s="2" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="149" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>334</v>
+        <v>436</v>
       </c>
       <c r="C149" s="5">
         <v>0</v>
       </c>
       <c r="D149" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="E149" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F149" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G149" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A150" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B150" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C150" s="5">
+        <v>0</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E150" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F150" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G150" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="E149" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F149" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G149" s="6" t="s">
-        <v>391</v>
-      </c>
-      <c r="H149" s="3" t="s">
+      <c r="H150" s="3" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+      <c r="A151" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="C151" s="5">
+        <v>1</v>
+      </c>
+      <c r="D151" s="5" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="150" spans="1:8" ht="145" x14ac:dyDescent="0.35">
-      <c r="A150" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C150" s="5">
+      <c r="E151" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F151" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G151" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="H151" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+      <c r="A152" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B152" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C152" s="5">
+        <v>0</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="E152" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F152" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G152" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="H152" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A153" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B153" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C153" s="5">
         <v>1</v>
       </c>
-      <c r="D150" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="E150" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F150" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G150" s="6" t="s">
+      <c r="D153" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="E153" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F153" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G153" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="H153" s="2" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A154" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B154" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="H150" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A151" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B151" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C151" s="5">
-        <v>0</v>
-      </c>
-      <c r="D151" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="E151" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G151" s="6" t="s">
-        <v>336</v>
-      </c>
-      <c r="H151" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A152" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B152" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C152" s="5">
-        <v>1</v>
-      </c>
-      <c r="D152" s="5" t="s">
+      <c r="C154" s="5">
+        <v>2</v>
+      </c>
+      <c r="D154" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="E152" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F152" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G152" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="H152" s="2" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A153" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B153" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C153" s="5">
-        <v>2</v>
-      </c>
-      <c r="D153" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="E153" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F153" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G153" s="6" t="s">
+      <c r="E154" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G154" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="H154" s="2" t="s">
         <v>458</v>
-      </c>
-      <c r="H153" s="2" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A154" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B154" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="C154" s="5">
-        <v>0</v>
-      </c>
-      <c r="D154" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="E154" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F154" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G154" s="6" t="s">
-        <v>341</v>
-      </c>
-      <c r="H154" s="2" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B155" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C155" s="5">
+        <v>0</v>
+      </c>
+      <c r="D155" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="C155" s="5">
+      <c r="E155" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G155" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="H155" s="2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A156" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B156" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C156" s="5">
         <v>1</v>
       </c>
-      <c r="D155" s="5" t="s">
+      <c r="D156" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="E156" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G156" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="E155" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F155" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G155" s="6" t="s">
+      <c r="H156" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="H155" s="3" t="s">
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A157" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C157" s="5">
+        <v>2</v>
+      </c>
+      <c r="D157" s="5" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A156" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="B156" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="C156" s="5">
-        <v>2</v>
-      </c>
-      <c r="D156" s="5" t="s">
+      <c r="E157" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G157" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="E156" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F156" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G156" s="6" t="s">
+      <c r="H157" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="H156" s="3" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="157" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A157" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="B157" s="5" t="s">
+    </row>
+    <row r="158" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A158" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="B158" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="C157" s="5">
+      <c r="C158" s="5">
         <v>1</v>
       </c>
-      <c r="D157" s="5" t="s">
+      <c r="D158" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G158" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="E157" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G157" s="6" t="s">
+      <c r="H158" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="H157" s="2" t="s">
-        <v>465</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added text for the tooltip to words and added icon to footer link.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2031E34-7659-4F9B-B844-4F598EF64059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2CB35E-E211-4FFB-9203-491C8E2A4EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5260" yWindow="2750" windowWidth="25060" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10040" yWindow="2530" windowWidth="25060" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8932,215 +8932,6 @@
     </r>
   </si>
   <si>
-    <t>5fb91df8d1db2e1a9a27b9be5d8a5c60</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Sign in**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) or [**create**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) an ILAO Easy Form account to **save your progress**.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Feedback, suggestions, or comments? [**Let us know**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">){:target='_blank'}.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if nav.get_section() != None:
-% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
-% if current_context().question_id == None:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif 'review screen' not in current_context().question_id:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif
-% endif
-% endif</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -10596,212 +10387,6 @@
 :bell: ¡Respuestas guardadas disponibles!  
 ${action_button_html(url_action('load_answer'), icon='folder-open', label='Respuestas guardadas', size='md' )}
 % endif</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Iniciar sesión**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) o [**crear**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) una cuenta de ILAO Easy Form para **guardar tu progreso**.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-¿Comentarios, sugerencias u observaciones? [**Cuéntanos**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">){:target='_blank'}.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if nav.get_section() != None:
-% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
-% if current_context().question_id == None:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif "review screen" not in current_context().question_id:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif
-% endif
-% endif</t>
-    </r>
   </si>
   <si>
     <t>No puedes continuar a menos que aceptes los Términos de uso y la Política de privacidad.</t>
@@ -11076,6 +10661,421 @@
       </rPr>
       <t>[NEWLINE]</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Sign in**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) or [**create**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) an ILAO Easy Form account to **save your progress**.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Feedback, suggestions, or comments? [**Let us know :external-link:**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">){:target='_blank'}.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if nav.get_section() != None:
+% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
+% if current_context().question_id == None:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif 'review screen' not in current_context().question_id:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif
+% endif
+% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Iniciar sesión**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) o [**crear**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) una cuenta de ILAO Easy Form para **guardar tu progreso**.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+¿Comentarios, sugerencias u observaciones? [**Cuéntanos :external-link:**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">){:target='_blank'}.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if nav.get_section() != None:
+% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
+% if current_context().question_id == None:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif "review screen" not in current_context().question_id:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif
+% endif
+% endif</t>
+    </r>
+  </si>
+  <si>
+    <t>d1644c7e85e7c5d8cffcd3168f9f0a26</t>
   </si>
 </sst>
 </file>
@@ -11587,7 +11587,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>459</v>
+        <v>507</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11596,10 +11596,10 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>482</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
@@ -11625,7 +11625,7 @@
         <v>365</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -11633,13 +11633,13 @@
         <v>368</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>8</v>
@@ -11648,10 +11648,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -11807,7 +11807,7 @@
         <v>58</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -11859,7 +11859,7 @@
         <v>355</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -11911,7 +11911,7 @@
         <v>356</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -11963,7 +11963,7 @@
         <v>357</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -12015,7 +12015,7 @@
         <v>358</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -12119,7 +12119,7 @@
         <v>42</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -12145,7 +12145,7 @@
         <v>44</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12353,7 +12353,7 @@
         <v>60</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -12639,7 +12639,7 @@
         <v>82</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
@@ -12743,7 +12743,7 @@
         <v>90</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
@@ -12795,7 +12795,7 @@
         <v>94</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -12991,7 +12991,7 @@
         <v>1</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>8</v>
@@ -13000,10 +13000,10 @@
         <v>9</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -13575,7 +13575,7 @@
         <v>159</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -13653,7 +13653,7 @@
         <v>166</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="195" customHeight="1" x14ac:dyDescent="0.35">
@@ -13705,7 +13705,7 @@
         <v>170</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="87" x14ac:dyDescent="0.35">
@@ -13731,7 +13731,7 @@
         <v>173</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -13757,7 +13757,7 @@
         <v>175</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -13783,12 +13783,12 @@
         <v>370</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>10</v>
@@ -13797,7 +13797,7 @@
         <v>1</v>
       </c>
       <c r="D89" s="5" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>8</v>
@@ -13806,10 +13806,10 @@
         <v>9</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.35">
@@ -13887,7 +13887,7 @@
         <v>183</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -14118,10 +14118,10 @@
         <v>9</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="87" x14ac:dyDescent="0.35">
@@ -14147,7 +14147,7 @@
         <v>353</v>
       </c>
       <c r="H102" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -14170,10 +14170,10 @@
         <v>9</v>
       </c>
       <c r="G103" s="6" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -14196,7 +14196,7 @@
         <v>9</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>260</v>
@@ -14222,7 +14222,7 @@
         <v>9</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="H105" s="3" t="s">
         <v>261</v>
@@ -14733,7 +14733,7 @@
         <v>1</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E125" s="5" t="s">
         <v>8</v>
@@ -14742,10 +14742,10 @@
         <v>9</v>
       </c>
       <c r="G125" s="6" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="H125" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.35">
@@ -14951,7 +14951,7 @@
         <v>403</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
@@ -14977,7 +14977,7 @@
         <v>405</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.35">
@@ -15467,7 +15467,7 @@
         <v>387</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
@@ -15585,19 +15585,19 @@
         <v>1</v>
       </c>
       <c r="D158" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G158" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="H158" s="2" t="s">
         <v>462</v>
-      </c>
-      <c r="E158" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F158" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G158" s="6" t="s">
-        <v>463</v>
-      </c>
-      <c r="H158" s="2" t="s">
-        <v>464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed remaining issues on the system screens
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38D3993-014F-4581-9B29-9786E3A035C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABB31AB-5DBA-4B01-BFDF-899CB0F47EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8290" yWindow="6810" windowWidth="30090" windowHeight="13520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13360" yWindow="6550" windowWidth="21910" windowHeight="13050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3613,15 +3613,6 @@
     </r>
   </si>
   <si>
-    <t>3932e7303b17dba216943212d78c6356</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thank you for your interest in Illinois Legal Aid Online **{Easy Forms}**.
-&lt;a target="_self" href="https://easyforms.illinoislegalaid.org/user/sign-in?next=https://easyforms.illinoislegalaid.org/interviews"&gt;Sign in&lt;/a&gt; to your ILAO Easy Forms account to access your saved Easy Forms.
-Looking for other forms? Check out the [**ILAO Form Library**](https://www.illinoislegalaid.org/form-library).
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">After you click **Next**, it may take a few moments to finish making your forms.
 ###### You do not need to refresh your screen. Hang in there!
@@ -3725,12 +3716,6 @@
     <t>docassemble.ILAO:ilao_interview_list.yml</t>
   </si>
   <si>
-    <t xml:space="preserve">Gracias por su interés en Illinois Legal Aid Online **{Formularios Fáciles}**.
-&lt;a target=""_self"" href=""https://easyforms.illinoislegalaid.org/user/sign-in?next=https://easyforms.illinoislegalaid.org/interviews""&gt;Inicie sesión&lt;/a&gt; en su cuenta de ILAO Formularios Fáciles para acceder a sus Formularios Fáciles guardados.
-¿Buscando otros formularios? Consulte la [**Biblioteca de Formularios de ILAO**](https://es.illinoislegalaid.org/form-library).
-</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -11268,6 +11253,113 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>ee894afce86460984c2e2ade5af8093b</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Thank you for your interest in Illinois Legal Aid Online **{Easy Forms}**.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;a target="_self" href="/user/sign-in"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sign in</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to your ILAO Easy Forms account to access your saved Easy Forms.
+Looking for other forms? Check out the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[**ILAO Form Library**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.illinoislegalaid.org/form-library</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Gracias por su interés en Illinois Legal Aid Online **{Formularios Fáciles}**.
+&lt;a target=""_self"" href=""/user/sign-in""&gt;Inicie sesión&lt;/a&gt; en su cuenta de ILAO Formularios Fáciles para acceder a sus Formularios Fáciles guardados.
+¿Buscando otros formularios? Consulte la [**Biblioteca de Formularios de ILAO**](https://es.illinoislegalaid.org/form-library).
+</t>
   </si>
 </sst>
 </file>
@@ -11352,7 +11444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -11375,6 +11467,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -11727,7 +11825,7 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>288</v>
@@ -11745,15 +11843,15 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>288</v>
@@ -11771,15 +11869,15 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>288</v>
@@ -11788,7 +11886,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11797,15 +11895,15 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>288</v>
@@ -11814,7 +11912,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>8</v>
@@ -11823,24 +11921,24 @@
         <v>9</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>8</v>
@@ -11849,24 +11947,24 @@
         <v>9</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11875,24 +11973,24 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>8</v>
@@ -11901,85 +11999,85 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>524</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>527</v>
-      </c>
       <c r="H9" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>528</v>
-      </c>
       <c r="H10" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>526</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>529</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>297</v>
@@ -11987,16 +12085,16 @@
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>8</v>
@@ -12005,24 +12103,24 @@
         <v>9</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>8</v>
@@ -12031,15 +12129,15 @@
         <v>9</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -12065,7 +12163,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -12083,15 +12181,15 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -12117,7 +12215,7 @@
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -12138,12 +12236,12 @@
         <v>54</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -12161,7 +12259,7 @@
         <v>9</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>223</v>
@@ -12169,7 +12267,7 @@
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -12190,12 +12288,12 @@
         <v>58</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -12221,7 +12319,7 @@
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -12239,15 +12337,15 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -12273,7 +12371,7 @@
     </row>
     <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -12291,15 +12389,15 @@
         <v>9</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -12325,7 +12423,7 @@
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -12343,15 +12441,15 @@
         <v>9</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -12377,7 +12475,7 @@
     </row>
     <row r="27" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -12395,15 +12493,15 @@
         <v>9</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -12429,7 +12527,7 @@
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -12455,7 +12553,7 @@
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -12481,7 +12579,7 @@
     </row>
     <row r="31" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -12502,12 +12600,12 @@
         <v>42</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -12528,12 +12626,12 @@
         <v>44</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -12559,7 +12657,7 @@
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -12585,7 +12683,7 @@
     </row>
     <row r="35" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -12611,7 +12709,7 @@
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -12637,7 +12735,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12658,12 +12756,12 @@
         <v>54</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12689,7 +12787,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12715,7 +12813,7 @@
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12736,12 +12834,12 @@
         <v>60</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12767,7 +12865,7 @@
     </row>
     <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12793,7 +12891,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12819,7 +12917,7 @@
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12845,7 +12943,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12871,7 +12969,7 @@
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12897,7 +12995,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12923,7 +13021,7 @@
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12949,7 +13047,7 @@
     </row>
     <row r="49" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12975,7 +13073,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -13001,7 +13099,7 @@
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -13022,12 +13120,12 @@
         <v>82</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -13053,7 +13151,7 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -13079,7 +13177,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -13105,7 +13203,7 @@
     </row>
     <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -13126,12 +13224,12 @@
         <v>90</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -13157,7 +13255,7 @@
     </row>
     <row r="57" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -13178,12 +13276,12 @@
         <v>94</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>14</v>
@@ -13209,7 +13307,7 @@
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>14</v>
@@ -13235,7 +13333,7 @@
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>14</v>
@@ -13261,7 +13359,7 @@
     </row>
     <row r="61" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>14</v>
@@ -13287,7 +13385,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>14</v>
@@ -13313,7 +13411,7 @@
     </row>
     <row r="63" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>14</v>
@@ -13339,7 +13437,7 @@
     </row>
     <row r="64" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A64" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>107</v>
@@ -13365,7 +13463,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>107</v>
@@ -13374,7 +13472,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>8</v>
@@ -13383,15 +13481,15 @@
         <v>9</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>110</v>
@@ -13417,7 +13515,7 @@
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>113</v>
@@ -13443,7 +13541,7 @@
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>113</v>
@@ -13469,7 +13567,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>113</v>
@@ -13495,7 +13593,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>113</v>
@@ -13521,7 +13619,7 @@
     </row>
     <row r="71" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>113</v>
@@ -13547,7 +13645,7 @@
     </row>
     <row r="72" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>113</v>
@@ -13573,16 +13671,16 @@
     </row>
     <row r="73" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>8</v>
@@ -13591,15 +13689,15 @@
         <v>9</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>12</v>
@@ -13625,7 +13723,7 @@
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>12</v>
@@ -13651,7 +13749,7 @@
     </row>
     <row r="76" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>12</v>
@@ -13677,7 +13775,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>12</v>
@@ -13703,7 +13801,7 @@
     </row>
     <row r="78" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A78" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>12</v>
@@ -13729,7 +13827,7 @@
     </row>
     <row r="79" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>12</v>
@@ -13755,7 +13853,7 @@
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>138</v>
@@ -13781,7 +13879,7 @@
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>138</v>
@@ -13807,7 +13905,7 @@
     </row>
     <row r="82" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>143</v>
@@ -13828,12 +13926,12 @@
         <v>145</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>143</v>
@@ -13859,7 +13957,7 @@
     </row>
     <row r="84" spans="1:8" ht="174" x14ac:dyDescent="0.35">
       <c r="A84" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>10</v>
@@ -13880,12 +13978,12 @@
         <v>149</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A85" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>150</v>
@@ -13911,7 +14009,7 @@
     </row>
     <row r="86" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A86" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>150</v>
@@ -13937,7 +14035,7 @@
     </row>
     <row r="87" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A87" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>155</v>
@@ -13963,7 +14061,7 @@
     </row>
     <row r="88" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>155</v>
@@ -13984,12 +14082,12 @@
         <v>159</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A89" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>160</v>
@@ -14015,7 +14113,7 @@
     </row>
     <row r="90" spans="1:8" ht="116" x14ac:dyDescent="0.35">
       <c r="A90" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>160</v>
@@ -14041,7 +14139,7 @@
     </row>
     <row r="91" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A91" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>160</v>
@@ -14062,12 +14160,12 @@
         <v>166</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>160</v>
@@ -14093,7 +14191,7 @@
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>160</v>
@@ -14114,12 +14212,12 @@
         <v>170</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A94" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>171</v>
@@ -14140,12 +14238,12 @@
         <v>173</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>171</v>
@@ -14166,12 +14264,12 @@
         <v>175</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>11</v>
@@ -14189,15 +14287,15 @@
         <v>9</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="5" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>10</v>
@@ -14206,7 +14304,7 @@
         <v>1</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>8</v>
@@ -14215,15 +14313,15 @@
         <v>9</v>
       </c>
       <c r="G97" s="6" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>11</v>
@@ -14249,7 +14347,7 @@
     </row>
     <row r="99" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A99" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>179</v>
@@ -14275,7 +14373,7 @@
     </row>
     <row r="100" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A100" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>179</v>
@@ -14296,12 +14394,12 @@
         <v>183</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>184</v>
@@ -14327,7 +14425,7 @@
     </row>
     <row r="102" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>184</v>
@@ -14353,7 +14451,7 @@
     </row>
     <row r="103" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>184</v>
@@ -14379,7 +14477,7 @@
     </row>
     <row r="104" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>184</v>
@@ -14405,7 +14503,7 @@
     </row>
     <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>184</v>
@@ -14431,7 +14529,7 @@
     </row>
     <row r="106" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>184</v>
@@ -14457,7 +14555,7 @@
     </row>
     <row r="107" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>197</v>
@@ -14483,7 +14581,7 @@
     </row>
     <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>197</v>
@@ -14509,7 +14607,7 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>202</v>
@@ -14527,15 +14625,15 @@
         <v>9</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A110" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>202</v>
@@ -14553,15 +14651,15 @@
         <v>9</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A111" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>205</v>
@@ -14579,15 +14677,15 @@
         <v>9</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A112" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>207</v>
@@ -14605,7 +14703,7 @@
         <v>9</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>260</v>
@@ -14613,7 +14711,7 @@
     </row>
     <row r="113" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A113" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>209</v>
@@ -14631,7 +14729,7 @@
         <v>9</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>261</v>
@@ -14639,7 +14737,7 @@
     </row>
     <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>211</v>
@@ -14657,15 +14755,15 @@
         <v>9</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A115" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>211</v>
@@ -14686,12 +14784,12 @@
         <v>214</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A116" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>215</v>
@@ -14717,7 +14815,7 @@
     </row>
     <row r="117" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A117" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>218</v>
@@ -14741,9 +14839,9 @@
         <v>348</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" ht="116" x14ac:dyDescent="0.35">
       <c r="A118" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>218</v>
@@ -14751,25 +14849,25 @@
       <c r="C118" s="5">
         <v>1</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="E118" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G118" s="6" t="s">
-        <v>352</v>
+      <c r="D118" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="E118" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F118" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G118" s="11" t="s">
+        <v>528</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>374</v>
+        <v>529</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>291</v>
@@ -14778,7 +14876,7 @@
         <v>0</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>8</v>
@@ -14787,15 +14885,15 @@
         <v>9</v>
       </c>
       <c r="G119" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="H119" s="2" t="s">
         <v>377</v>
-      </c>
-      <c r="H119" s="2" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>291</v>
@@ -14804,24 +14902,24 @@
         <v>1</v>
       </c>
       <c r="D120" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G120" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="H120" s="2" t="s">
         <v>378</v>
-      </c>
-      <c r="E120" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G120" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="H120" s="2" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A121" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>291</v>
@@ -14847,7 +14945,7 @@
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>294</v>
@@ -14873,7 +14971,7 @@
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>294</v>
@@ -14894,12 +14992,12 @@
         <v>299</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>294</v>
@@ -14920,12 +15018,12 @@
         <v>301</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>294</v>
@@ -14946,12 +15044,12 @@
         <v>303</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>294</v>
@@ -14977,7 +15075,7 @@
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B127" s="5" t="s">
         <v>294</v>
@@ -15003,7 +15101,7 @@
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>294</v>
@@ -15029,7 +15127,7 @@
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B129" s="5" t="s">
         <v>294</v>
@@ -15055,7 +15153,7 @@
     </row>
     <row r="130" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B130" s="5" t="s">
         <v>316</v>
@@ -15076,12 +15174,12 @@
         <v>318</v>
       </c>
       <c r="H130" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B131" s="5" t="s">
         <v>319</v>
@@ -15107,7 +15205,7 @@
     </row>
     <row r="132" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>11</v>
@@ -15133,7 +15231,7 @@
     </row>
     <row r="133" spans="1:8" ht="232" x14ac:dyDescent="0.35">
       <c r="A133" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>11</v>
@@ -15142,7 +15240,7 @@
         <v>1</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>8</v>
@@ -15151,15 +15249,15 @@
         <v>9</v>
       </c>
       <c r="G133" s="6" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>11</v>
@@ -15185,7 +15283,7 @@
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>11</v>
@@ -15211,16 +15309,16 @@
     </row>
     <row r="136" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A136" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C136" s="5">
         <v>0</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>8</v>
@@ -15229,24 +15327,24 @@
         <v>9</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="H136" s="8" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A137" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C137" s="5">
         <v>1</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>8</v>
@@ -15255,24 +15353,24 @@
         <v>9</v>
       </c>
       <c r="G137" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C138" s="5">
         <v>2</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>8</v>
@@ -15281,15 +15379,15 @@
         <v>9</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B139" s="5" t="s">
         <v>333</v>
@@ -15298,7 +15396,7 @@
         <v>0</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>8</v>
@@ -15307,13 +15405,13 @@
         <v>9</v>
       </c>
       <c r="G139" s="6" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="H139" s="7"/>
     </row>
     <row r="140" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B140" s="5" t="s">
         <v>333</v>
@@ -15322,7 +15420,7 @@
         <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>8</v>
@@ -15331,15 +15429,15 @@
         <v>9</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A141" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B141" s="5" t="s">
         <v>333</v>
@@ -15348,7 +15446,7 @@
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>8</v>
@@ -15357,15 +15455,15 @@
         <v>9</v>
       </c>
       <c r="G141" s="6" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A142" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B142" s="5" t="s">
         <v>333</v>
@@ -15374,7 +15472,7 @@
         <v>3</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>8</v>
@@ -15383,15 +15481,15 @@
         <v>9</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B143" s="5" t="s">
         <v>171</v>
@@ -15400,7 +15498,7 @@
         <v>0</v>
       </c>
       <c r="D143" s="5" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>8</v>
@@ -15409,13 +15507,13 @@
         <v>9</v>
       </c>
       <c r="G143" s="6" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="H143" s="7"/>
     </row>
     <row r="144" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A144" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B144" s="5" t="s">
         <v>171</v>
@@ -15424,7 +15522,7 @@
         <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E144" s="5" t="s">
         <v>8</v>
@@ -15433,15 +15531,15 @@
         <v>9</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A145" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B145" s="5" t="s">
         <v>171</v>
@@ -15450,7 +15548,7 @@
         <v>2</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>8</v>
@@ -15459,15 +15557,15 @@
         <v>9</v>
       </c>
       <c r="G145" s="6" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="H145" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B146" s="5" t="s">
         <v>171</v>
@@ -15476,7 +15574,7 @@
         <v>3</v>
       </c>
       <c r="D146" s="5" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>8</v>
@@ -15485,15 +15583,15 @@
         <v>9</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>171</v>
@@ -15502,7 +15600,7 @@
         <v>4</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>8</v>
@@ -15511,24 +15609,24 @@
         <v>9</v>
       </c>
       <c r="G147" s="6" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="H147" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C148" s="5">
         <v>0</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>8</v>
@@ -15537,22 +15635,22 @@
         <v>9</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="H148" s="7"/>
     </row>
     <row r="149" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A149" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C149" s="5">
         <v>1</v>
       </c>
       <c r="D149" s="5" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>8</v>
@@ -15561,24 +15659,24 @@
         <v>9</v>
       </c>
       <c r="G149" s="6" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="H149" s="2" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A150" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C150" s="5">
         <v>2</v>
       </c>
       <c r="D150" s="5" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>8</v>
@@ -15587,24 +15685,24 @@
         <v>9</v>
       </c>
       <c r="G150" s="6" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A151" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C151" s="5">
         <v>0</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E151" s="5" t="s">
         <v>8</v>
@@ -15613,24 +15711,24 @@
         <v>9</v>
       </c>
       <c r="G151" s="6" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A152" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C152" s="5">
         <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>8</v>
@@ -15639,24 +15737,24 @@
         <v>9</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A153" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C153" s="5">
         <v>2</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="E153" s="5" t="s">
         <v>8</v>
@@ -15665,15 +15763,15 @@
         <v>9</v>
       </c>
       <c r="G153" s="6" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A154" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B154" s="5" t="s">
         <v>338</v>
@@ -15682,7 +15780,7 @@
         <v>0</v>
       </c>
       <c r="D154" s="5" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="E154" s="5" t="s">
         <v>8</v>
@@ -15691,15 +15789,15 @@
         <v>9</v>
       </c>
       <c r="G154" s="6" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A155" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B155" s="5" t="s">
         <v>338</v>
@@ -15708,7 +15806,7 @@
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E155" s="5" t="s">
         <v>8</v>
@@ -15717,15 +15815,15 @@
         <v>9</v>
       </c>
       <c r="G155" s="6" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="H155" s="2" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B156" s="5" t="s">
         <v>338</v>
@@ -15734,7 +15832,7 @@
         <v>2</v>
       </c>
       <c r="D156" s="5" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="E156" s="5" t="s">
         <v>8</v>
@@ -15743,24 +15841,24 @@
         <v>9</v>
       </c>
       <c r="G156" s="6" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="H156" s="2" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A157" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C157" s="5">
         <v>0</v>
       </c>
       <c r="D157" s="5" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="E157" s="5" t="s">
         <v>8</v>
@@ -15769,15 +15867,15 @@
         <v>9</v>
       </c>
       <c r="G157" s="6" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A158" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B158" s="5" t="s">
         <v>333</v>
@@ -15786,7 +15884,7 @@
         <v>0</v>
       </c>
       <c r="D158" s="5" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="E158" s="5" t="s">
         <v>8</v>
@@ -15795,7 +15893,7 @@
         <v>9</v>
       </c>
       <c r="G158" s="6" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="H158" s="3" t="s">
         <v>330</v>
@@ -15803,7 +15901,7 @@
     </row>
     <row r="159" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A159" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B159" s="5" t="s">
         <v>329</v>
@@ -15824,12 +15922,12 @@
         <v>332</v>
       </c>
       <c r="H159" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A160" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B160" s="5" t="s">
         <v>333</v>
@@ -15850,12 +15948,12 @@
         <v>335</v>
       </c>
       <c r="H160" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A161" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B161" s="5" t="s">
         <v>333</v>
@@ -15873,15 +15971,15 @@
         <v>9</v>
       </c>
       <c r="G161" s="6" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="H161" s="2" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A162" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B162" s="5" t="s">
         <v>333</v>
@@ -15899,15 +15997,15 @@
         <v>9</v>
       </c>
       <c r="G162" s="6" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A163" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B163" s="5" t="s">
         <v>338</v>
@@ -15933,7 +16031,7 @@
     </row>
     <row r="164" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B164" s="5" t="s">
         <v>338</v>
@@ -15959,7 +16057,7 @@
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A165" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B165" s="5" t="s">
         <v>338</v>
@@ -15985,7 +16083,7 @@
     </row>
     <row r="166" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A166" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B166" s="5" t="s">
         <v>215</v>
@@ -15994,7 +16092,7 @@
         <v>1</v>
       </c>
       <c r="D166" s="5" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E166" s="5" t="s">
         <v>8</v>
@@ -16003,10 +16101,10 @@
         <v>9</v>
       </c>
       <c r="G166" s="6" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>